<commit_message>
Table S1: add per-treatment sign-flip counts and log-scale robustness results
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T86"/>
+  <dimension ref="A1:Y86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -445,12 +445,17 @@
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="28" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table S1. Per-treatment statistics for the 83 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; tolerance 0.2), and years to first detection of a significant trend (directional treatments only).</t>
+          <t>Table S1. Per-treatment statistics for the 83 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; tolerance 0.2), years to first detection of a significant trend (directional treatments only), the number, percentage (of consecutive measurement transitions), and years of sign flips, and the P-value and directional call when the trend analysis is repeated on the log response ratio.</t>
         </is>
       </c>
     </row>
@@ -555,6 +560,31 @@
           <t>Years to Detect</t>
         </is>
       </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>N Sign Flips</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>Sign Flip %</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>Flip Years</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>Log-scale P-value</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>Log-scale Directional Call</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -635,6 +665,25 @@
       <c r="T4" t="n">
         <v>12</v>
       </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>0.0436</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -715,6 +764,25 @@
       <c r="T5" t="n">
         <v>12</v>
       </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X5" t="n">
+        <v>0.082</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -797,6 +865,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X6" t="n">
+        <v>0.3015</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -877,6 +964,25 @@
       <c r="T7" t="n">
         <v>1.9986</v>
       </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>0.4746</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -959,6 +1065,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U8" t="n">
+        <v>4</v>
+      </c>
+      <c r="V8" t="n">
+        <v>36.3636</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>2010; 2014; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X8" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>decreasing</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1041,6 +1166,23 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U9" t="n">
+        <v>1</v>
+      </c>
+      <c r="V9" t="n">
+        <v>9.0909</v>
+      </c>
+      <c r="W9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.3927</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1123,6 +1265,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>0.4628</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1203,6 +1364,25 @@
       <c r="T11" t="n">
         <v>16</v>
       </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>0.0447</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>decreasing</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1283,6 +1463,25 @@
       <c r="T12" t="n">
         <v>8</v>
       </c>
+      <c r="U12" t="n">
+        <v>2</v>
+      </c>
+      <c r="V12" t="n">
+        <v>18.1818</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>2019; 2021</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>0.6172</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1363,6 +1562,25 @@
       <c r="T13" t="n">
         <v>12</v>
       </c>
+      <c r="U13" t="n">
+        <v>6</v>
+      </c>
+      <c r="V13" t="n">
+        <v>46.1538</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>2013; 2014; 2015; 2016; 2020; 2021</t>
+        </is>
+      </c>
+      <c r="X13" t="n">
+        <v>0.5968</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1445,6 +1663,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X14" t="n">
+        <v>0.8399</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1527,6 +1764,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U15" t="n">
+        <v>2</v>
+      </c>
+      <c r="V15" t="n">
+        <v>22.2222</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>2020; 2021</t>
+        </is>
+      </c>
+      <c r="X15" t="n">
+        <v>0.2925</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1609,6 +1865,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X16" t="n">
+        <v>0.7542</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1691,6 +1966,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U17" t="n">
+        <v>3</v>
+      </c>
+      <c r="V17" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>2015; 2016; 2021</t>
+        </is>
+      </c>
+      <c r="X17" t="n">
+        <v>0.4578</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1773,6 +2067,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X18" t="n">
+        <v>0.8691</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1853,6 +2166,25 @@
       <c r="T19" t="n">
         <v>2.9979</v>
       </c>
+      <c r="U19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>decreasing</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1933,6 +2265,25 @@
       <c r="T20" t="n">
         <v>12</v>
       </c>
+      <c r="U20" t="n">
+        <v>2</v>
+      </c>
+      <c r="V20" t="n">
+        <v>9.0909</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>1999; 2007</t>
+        </is>
+      </c>
+      <c r="X20" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2015,6 +2366,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U21" t="n">
+        <v>6</v>
+      </c>
+      <c r="V21" t="n">
+        <v>26.087</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>2000; 2001; 2009; 2010; 2020; 2021</t>
+        </is>
+      </c>
+      <c r="X21" t="n">
+        <v>0.4972</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2095,6 +2465,25 @@
       <c r="T22" t="n">
         <v>10.0014</v>
       </c>
+      <c r="U22" t="n">
+        <v>2</v>
+      </c>
+      <c r="V22" t="n">
+        <v>15.3846</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>2015; 2019</t>
+        </is>
+      </c>
+      <c r="X22" t="n">
+        <v>0.2823</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2175,6 +2564,25 @@
       <c r="T23" t="n">
         <v>4</v>
       </c>
+      <c r="U23" t="n">
+        <v>2</v>
+      </c>
+      <c r="V23" t="n">
+        <v>22.2222</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>2014; 2020</t>
+        </is>
+      </c>
+      <c r="X23" t="n">
+        <v>0.9277</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2257,6 +2665,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U24" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X24" t="n">
+        <v>0.8292</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2339,6 +2766,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X25" t="n">
+        <v>0.6636</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2421,6 +2867,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U26" t="n">
+        <v>3</v>
+      </c>
+      <c r="V26" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>2015; 2016; 2021</t>
+        </is>
+      </c>
+      <c r="X26" t="n">
+        <v>0.411</v>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2503,6 +2968,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U27" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X27" t="n">
+        <v>0.6061</v>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2585,6 +3069,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U28" t="n">
+        <v>4</v>
+      </c>
+      <c r="V28" t="n">
+        <v>50</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>2014; 2017; 2018; 2020</t>
+        </is>
+      </c>
+      <c r="X28" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2665,6 +3168,25 @@
       <c r="T29" t="n">
         <v>15.0007</v>
       </c>
+      <c r="U29" t="n">
+        <v>3</v>
+      </c>
+      <c r="V29" t="n">
+        <v>13.6364</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>2000; 2005; 2021</t>
+        </is>
+      </c>
+      <c r="X29" t="n">
+        <v>0.0138</v>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2745,6 +3267,25 @@
       <c r="T30" t="n">
         <v>7.0007</v>
       </c>
+      <c r="U30" t="n">
+        <v>11</v>
+      </c>
+      <c r="V30" t="n">
+        <v>47.8261</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>1999; 2000; 2001; 2009; 2011; 2012; 2014; 2015; 2016; 2020; 2021</t>
+        </is>
+      </c>
+      <c r="X30" t="n">
+        <v>0.9114</v>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2825,6 +3366,25 @@
       <c r="T31" t="n">
         <v>3.0007</v>
       </c>
+      <c r="U31" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X31" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>decreasing</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2907,6 +3467,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U32" t="n">
+        <v>6</v>
+      </c>
+      <c r="V32" t="n">
+        <v>66.66670000000001</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>2013; 2014; 2015; 2018; 2019; 2021</t>
+        </is>
+      </c>
+      <c r="X32" t="n">
+        <v>0.6485</v>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2989,6 +3568,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X33" t="n">
+        <v>0.2604</v>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3071,6 +3669,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U34" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X34" t="n">
+        <v>0.3381</v>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3153,6 +3770,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U35" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X35" t="n">
+        <v>0.2936</v>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3233,6 +3869,23 @@
       <c r="T36" t="n">
         <v>2.0014</v>
       </c>
+      <c r="U36" t="n">
+        <v>1</v>
+      </c>
+      <c r="V36" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="W36" t="n">
+        <v>2021</v>
+      </c>
+      <c r="X36" t="n">
+        <v>0.8378</v>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3313,6 +3966,25 @@
       <c r="T37" t="n">
         <v>13.9986</v>
       </c>
+      <c r="U37" t="n">
+        <v>6</v>
+      </c>
+      <c r="V37" t="n">
+        <v>27.2727</v>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>2000; 2004; 2009; 2010; 2015; 2016</t>
+        </is>
+      </c>
+      <c r="X37" t="n">
+        <v>0.0047</v>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3395,6 +4067,23 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U38" t="n">
+        <v>1</v>
+      </c>
+      <c r="V38" t="n">
+        <v>4.3478</v>
+      </c>
+      <c r="W38" t="n">
+        <v>2020</v>
+      </c>
+      <c r="X38" t="n">
+        <v>0.4208</v>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3477,6 +4166,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X39" t="n">
+        <v>0.7864</v>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3559,6 +4267,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" t="n">
+        <v>0</v>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X40" t="n">
+        <v>0.4956</v>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3639,6 +4366,25 @@
       <c r="T41" t="n">
         <v>9.0021</v>
       </c>
+      <c r="U41" t="n">
+        <v>0</v>
+      </c>
+      <c r="V41" t="n">
+        <v>0</v>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X41" t="n">
+        <v>0.0266</v>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>decreasing</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3721,6 +4467,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U42" t="n">
+        <v>0</v>
+      </c>
+      <c r="V42" t="n">
+        <v>0</v>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X42" t="n">
+        <v>0.438</v>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3803,6 +4568,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" t="n">
+        <v>0</v>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X43" t="n">
+        <v>0.8431999999999999</v>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3885,6 +4669,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
+      <c r="V44" t="n">
+        <v>0</v>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X44" t="n">
+        <v>0.2542</v>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3965,6 +4768,25 @@
       <c r="T45" t="n">
         <v>13.9986</v>
       </c>
+      <c r="U45" t="n">
+        <v>4</v>
+      </c>
+      <c r="V45" t="n">
+        <v>18.1818</v>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>2000; 2004; 2018; 2019</t>
+        </is>
+      </c>
+      <c r="X45" t="n">
+        <v>0.0539</v>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4045,6 +4867,25 @@
       <c r="T46" t="n">
         <v>3.0007</v>
       </c>
+      <c r="U46" t="n">
+        <v>0</v>
+      </c>
+      <c r="V46" t="n">
+        <v>0</v>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X46" t="n">
+        <v>0.1158</v>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4127,6 +4968,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U47" t="n">
+        <v>2</v>
+      </c>
+      <c r="V47" t="n">
+        <v>40</v>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>2020; 2021</t>
+        </is>
+      </c>
+      <c r="X47" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4207,6 +5067,23 @@
       <c r="T48" t="n">
         <v>8</v>
       </c>
+      <c r="U48" t="n">
+        <v>1</v>
+      </c>
+      <c r="V48" t="n">
+        <v>8.333299999999999</v>
+      </c>
+      <c r="W48" t="n">
+        <v>2016</v>
+      </c>
+      <c r="X48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4287,6 +5164,25 @@
       <c r="T49" t="n">
         <v>12</v>
       </c>
+      <c r="U49" t="n">
+        <v>3</v>
+      </c>
+      <c r="V49" t="n">
+        <v>25</v>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>2017; 2020; 2021</t>
+        </is>
+      </c>
+      <c r="X49" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4367,6 +5263,25 @@
       <c r="T50" t="n">
         <v>4.9993</v>
       </c>
+      <c r="U50" t="n">
+        <v>0</v>
+      </c>
+      <c r="V50" t="n">
+        <v>0</v>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X50" t="n">
+        <v>0.7884</v>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4447,6 +5362,25 @@
       <c r="T51" t="n">
         <v>7.0007</v>
       </c>
+      <c r="U51" t="n">
+        <v>9</v>
+      </c>
+      <c r="V51" t="n">
+        <v>30</v>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>1999; 2003; 2004; 2006; 2010; 2011; 2014; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X51" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>decreasing</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4529,6 +5463,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U52" t="n">
+        <v>7</v>
+      </c>
+      <c r="V52" t="n">
+        <v>21.875</v>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>1991; 1999; 2001; 2006; 2007; 2018; 2019</t>
+        </is>
+      </c>
+      <c r="X52" t="n">
+        <v>0.1141</v>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4609,6 +5562,25 @@
       <c r="T53" t="n">
         <v>32</v>
       </c>
+      <c r="U53" t="n">
+        <v>6</v>
+      </c>
+      <c r="V53" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>1994; 1995; 1999; 2000; 2018; 2019</t>
+        </is>
+      </c>
+      <c r="X53" t="n">
+        <v>0.0465</v>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4691,6 +5663,23 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U54" t="n">
+        <v>1</v>
+      </c>
+      <c r="V54" t="n">
+        <v>50</v>
+      </c>
+      <c r="W54" t="n">
+        <v>1995</v>
+      </c>
+      <c r="X54" t="n">
+        <v>0.7694</v>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4771,6 +5760,25 @@
       <c r="T55" t="n">
         <v>24</v>
       </c>
+      <c r="U55" t="n">
+        <v>8</v>
+      </c>
+      <c r="V55" t="n">
+        <v>25</v>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>1991; 1992; 1994; 1995; 1999; 2001; 2018; 2019</t>
+        </is>
+      </c>
+      <c r="X55" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4851,6 +5859,25 @@
       <c r="T56" t="n">
         <v>32</v>
       </c>
+      <c r="U56" t="n">
+        <v>15</v>
+      </c>
+      <c r="V56" t="n">
+        <v>50</v>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>1992; 1993; 1998; 1999; 2003; 2005; 2006; 2007; 2010; 2011; 2012; 2014; 2016; 2017; 2022</t>
+        </is>
+      </c>
+      <c r="X56" t="n">
+        <v>0.0557</v>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4931,6 +5958,25 @@
       <c r="T57" t="n">
         <v>7.0007</v>
       </c>
+      <c r="U57" t="n">
+        <v>11</v>
+      </c>
+      <c r="V57" t="n">
+        <v>33.3333</v>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>1999; 2000; 2002; 2003; 2005; 2006; 2007; 2010; 2012; 2013; 2014</t>
+        </is>
+      </c>
+      <c r="X57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5011,6 +6057,25 @@
       <c r="T58" t="n">
         <v>5.9986</v>
       </c>
+      <c r="U58" t="n">
+        <v>9</v>
+      </c>
+      <c r="V58" t="n">
+        <v>25.7143</v>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>1987; 1989; 1990; 2000; 2001; 2006; 2007; 2016; 2017</t>
+        </is>
+      </c>
+      <c r="X58" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5091,6 +6156,25 @@
       <c r="T59" t="n">
         <v>3.0007</v>
       </c>
+      <c r="U59" t="n">
+        <v>9</v>
+      </c>
+      <c r="V59" t="n">
+        <v>25.7143</v>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>1988; 2000; 2001; 2006; 2007; 2016; 2017; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X59" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5171,6 +6255,25 @@
       <c r="T60" t="n">
         <v>7.0007</v>
       </c>
+      <c r="U60" t="n">
+        <v>11</v>
+      </c>
+      <c r="V60" t="n">
+        <v>33.3333</v>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>1999; 2000; 2002; 2003; 2005; 2006; 2007; 2011; 2012; 2013; 2014</t>
+        </is>
+      </c>
+      <c r="X60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5251,6 +6354,25 @@
       <c r="T61" t="n">
         <v>28.9993</v>
       </c>
+      <c r="U61" t="n">
+        <v>15</v>
+      </c>
+      <c r="V61" t="n">
+        <v>42.8571</v>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>1987; 1996; 1997; 2000; 2002; 2003; 2005; 2006; 2007; 2013; 2014; 2016; 2017; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X61" t="n">
+        <v>0.3215</v>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5331,6 +6453,25 @@
       <c r="T62" t="n">
         <v>7.0007</v>
       </c>
+      <c r="U62" t="n">
+        <v>6</v>
+      </c>
+      <c r="V62" t="n">
+        <v>17.1429</v>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>2000; 2001; 2006; 2007; 2016; 2017</t>
+        </is>
+      </c>
+      <c r="X62" t="n">
+        <v>0.4585</v>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5411,6 +6552,25 @@
       <c r="T63" t="n">
         <v>4.9993</v>
       </c>
+      <c r="U63" t="n">
+        <v>6</v>
+      </c>
+      <c r="V63" t="n">
+        <v>17.1429</v>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>2000; 2001; 2006; 2007; 2016; 2017</t>
+        </is>
+      </c>
+      <c r="X63" t="n">
+        <v>0.4876</v>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5491,6 +6651,25 @@
       <c r="T64" t="n">
         <v>31.0007</v>
       </c>
+      <c r="U64" t="n">
+        <v>21</v>
+      </c>
+      <c r="V64" t="n">
+        <v>60</v>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>1987; 1988; 1990; 1991; 1992; 1994; 1995; 1996; 1999; 2000; 2002; 2006; 2007; 2010; 2012; 2013; 2014; 2016; 2017; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X64" t="n">
+        <v>0.0977</v>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5571,6 +6750,25 @@
       <c r="T65" t="n">
         <v>5.9986</v>
       </c>
+      <c r="U65" t="n">
+        <v>11</v>
+      </c>
+      <c r="V65" t="n">
+        <v>31.4286</v>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>2005; 2006; 2007; 2009; 2012; 2013; 2014; 2016; 2017; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X65" t="n">
+        <v>0.0166</v>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5651,6 +6849,25 @@
       <c r="T66" t="n">
         <v>5.9986</v>
       </c>
+      <c r="U66" t="n">
+        <v>19</v>
+      </c>
+      <c r="V66" t="n">
+        <v>54.2857</v>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>1987; 1988; 1989; 1994; 1996; 2000; 2001; 2003; 2004; 2006; 2007; 2011; 2012; 2013; 2014; 2016; 2017; 2018; 2020</t>
+        </is>
+      </c>
+      <c r="X66" t="n">
+        <v>0.4726</v>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5731,6 +6948,25 @@
       <c r="T67" t="n">
         <v>4.9993</v>
       </c>
+      <c r="U67" t="n">
+        <v>17</v>
+      </c>
+      <c r="V67" t="n">
+        <v>48.5714</v>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>1987; 1988; 1989; 1994; 1996; 2000; 2001; 2006; 2007; 2010; 2011; 2013; 2014; 2016; 2017; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X67" t="n">
+        <v>0.2281</v>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5811,6 +7047,25 @@
       <c r="T68" t="n">
         <v>4</v>
       </c>
+      <c r="U68" t="n">
+        <v>15</v>
+      </c>
+      <c r="V68" t="n">
+        <v>42.8571</v>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>1999; 2000; 2001; 2003; 2004; 2006; 2007; 2009; 2012; 2013; 2014; 2016; 2017; 2019; 2020</t>
+        </is>
+      </c>
+      <c r="X68" t="n">
+        <v>0.0098</v>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5891,6 +7146,25 @@
       <c r="T69" t="n">
         <v>5.9986</v>
       </c>
+      <c r="U69" t="n">
+        <v>12</v>
+      </c>
+      <c r="V69" t="n">
+        <v>34.2857</v>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>1987; 2000; 2001; 2006; 2007; 2009; 2012; 2013; 2014; 2016; 2017; 2019</t>
+        </is>
+      </c>
+      <c r="X69" t="n">
+        <v>0.0653</v>
+      </c>
+      <c r="Y69" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5971,6 +7245,25 @@
       <c r="T70" t="n">
         <v>4</v>
       </c>
+      <c r="U70" t="n">
+        <v>12</v>
+      </c>
+      <c r="V70" t="n">
+        <v>34.2857</v>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>1987; 2000; 2001; 2006; 2007; 2009; 2012; 2013; 2014; 2016; 2017; 2019</t>
+        </is>
+      </c>
+      <c r="X70" t="n">
+        <v>0.0261</v>
+      </c>
+      <c r="Y70" t="inlineStr">
+        <is>
+          <t>decreasing</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6051,6 +7344,25 @@
       <c r="T71" t="n">
         <v>28</v>
       </c>
+      <c r="U71" t="n">
+        <v>18</v>
+      </c>
+      <c r="V71" t="n">
+        <v>51.4286</v>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>1988; 1989; 1990; 1991; 1996; 1997; 1999; 2001; 2004; 2005; 2006; 2007; 2009; 2012; 2016; 2017; 2019; 2021</t>
+        </is>
+      </c>
+      <c r="X71" t="n">
+        <v>0.7178</v>
+      </c>
+      <c r="Y71" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6133,6 +7445,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U72" t="n">
+        <v>0</v>
+      </c>
+      <c r="V72" t="n">
+        <v>0</v>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X72" t="n">
+        <v>0.716</v>
+      </c>
+      <c r="Y72" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6213,6 +7544,25 @@
       <c r="T73" t="n">
         <v>3.0007</v>
       </c>
+      <c r="U73" t="n">
+        <v>2</v>
+      </c>
+      <c r="V73" t="n">
+        <v>33.3333</v>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>2008; 2009</t>
+        </is>
+      </c>
+      <c r="X73" t="n">
+        <v>0.7323</v>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6293,6 +7643,25 @@
       <c r="T74" t="n">
         <v>2.0014</v>
       </c>
+      <c r="U74" t="n">
+        <v>2</v>
+      </c>
+      <c r="V74" t="n">
+        <v>33.3333</v>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>2007; 2008</t>
+        </is>
+      </c>
+      <c r="X74" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6375,6 +7744,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U75" t="n">
+        <v>0</v>
+      </c>
+      <c r="V75" t="n">
+        <v>0</v>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X75" t="n">
+        <v>0.0426</v>
+      </c>
+      <c r="Y75" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6457,6 +7845,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U76" t="n">
+        <v>0</v>
+      </c>
+      <c r="V76" t="n">
+        <v>0</v>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X76" t="n">
+        <v>0.1891</v>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6537,6 +7944,23 @@
       <c r="T77" t="n">
         <v>6.0014</v>
       </c>
+      <c r="U77" t="n">
+        <v>1</v>
+      </c>
+      <c r="V77" t="n">
+        <v>25</v>
+      </c>
+      <c r="W77" t="n">
+        <v>2007</v>
+      </c>
+      <c r="X77" t="n">
+        <v>0.1006</v>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6619,6 +8043,23 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U78" t="n">
+        <v>1</v>
+      </c>
+      <c r="V78" t="n">
+        <v>25</v>
+      </c>
+      <c r="W78" t="n">
+        <v>2007</v>
+      </c>
+      <c r="X78" t="n">
+        <v>0.2231</v>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6699,6 +8140,23 @@
       <c r="T79" t="n">
         <v>6.0014</v>
       </c>
+      <c r="U79" t="n">
+        <v>1</v>
+      </c>
+      <c r="V79" t="n">
+        <v>25</v>
+      </c>
+      <c r="W79" t="n">
+        <v>2007</v>
+      </c>
+      <c r="X79" t="n">
+        <v>0.1405</v>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6781,6 +8239,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U80" t="n">
+        <v>0</v>
+      </c>
+      <c r="V80" t="n">
+        <v>0</v>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X80" t="n">
+        <v>0.5039</v>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6861,6 +8338,25 @@
       <c r="T81" t="n">
         <v>4.9993</v>
       </c>
+      <c r="U81" t="n">
+        <v>2</v>
+      </c>
+      <c r="V81" t="n">
+        <v>16.6667</v>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>2007; 2008</t>
+        </is>
+      </c>
+      <c r="X81" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6943,6 +8439,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U82" t="n">
+        <v>8</v>
+      </c>
+      <c r="V82" t="n">
+        <v>50</v>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>2006; 2007; 2013; 2014; 2015; 2016; 2018; 2019</t>
+        </is>
+      </c>
+      <c r="X82" t="n">
+        <v>0.8786</v>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7025,6 +8540,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U83" t="n">
+        <v>0</v>
+      </c>
+      <c r="V83" t="n">
+        <v>0</v>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X83" t="n">
+        <v>0.6223</v>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7105,6 +8639,25 @@
       <c r="T84" t="n">
         <v>4</v>
       </c>
+      <c r="U84" t="n">
+        <v>4</v>
+      </c>
+      <c r="V84" t="n">
+        <v>30.7692</v>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>2012; 2015; 2018; 2020</t>
+        </is>
+      </c>
+      <c r="X84" t="n">
+        <v>0.3646</v>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7187,6 +8740,25 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="U85" t="n">
+        <v>2</v>
+      </c>
+      <c r="V85" t="n">
+        <v>10.5263</v>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>2018; 2022</t>
+        </is>
+      </c>
+      <c r="X85" t="n">
+        <v>0.2031</v>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>non-directional</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7266,6 +8838,25 @@
       </c>
       <c r="T86" t="n">
         <v>5.9986</v>
+      </c>
+      <c r="U86" t="n">
+        <v>5</v>
+      </c>
+      <c r="V86" t="n">
+        <v>33.3333</v>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>1997; 1998; 2000; 2002; 2004</t>
+        </is>
+      </c>
+      <c r="X86" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>increasing</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Number supplementary tables in order of first citation
S1 = case-study details, S2 = per-treatment statistics, S3 = SiZer results.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -422,6 +422,1247 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Table S1. Details of the 18 case-study datasets: setting, experiment, manipulation, response variable and type, years analyzed, number of years sampled, number of analyzable treatments (in parentheses, the number screened), EDI data-package identifier, and data citation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Site Name</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Ecosystem Type</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Manipulation</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Response Variable</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Response Type</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Years Analyzed</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>N Years Sampled</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>N Treatments</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>EDI Package</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Data Citation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GCE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Georgia Coastal Ecosystems</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Salt marsh</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Coastal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Tidal marsh disturbance experiment (PLT-GCED-2207)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Vegetation removal (disturbance)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Vegetation cover (%; carbon proxy)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2010-2020</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>knb-lter-gce.786.13</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Pennings, S. C. (2022). Data from: “Critical slowing down: vegetation height, cover and composition assess resilience of tidal fresh, brackish and salt marshes following experimental disturbance at twelve sites across the estuarine landscape ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/6df40a30859a7293db9a76fc4fff8cec</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PIE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plum Island Ecosystems</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Salt marsh creek</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Coastal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TIDE nutrient-enrichment experiment</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Fertilization (NO3)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Plant shoot mass</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2004-2020</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>knb-lter-pie.202.5</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Deegan, L., Warren, S. &amp; Mozdzer, T. (2022). Data from: “Marsh plant species shoot height, weight and diameters for Rowley River tidal creeks associated with long term fertilization experiments, Rowley and Ipswich, MA. ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/226fb7db2c7b9f8119e40c937b1a19a0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SBC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Santa Barbara Coastal</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kelp forest reef</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Coastal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Long-term kelp removal experiment</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Vegetation removal (annual and continual kelp removal)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Algal dry biomass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2008-2023</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>knb-lter-sbc.119.13</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Reed, D. C. &amp; Miller, R. J. (2024). Data from: “SBC LTER: Reef: Long-term experiment: biomass of kelp forest species, ongoing since 2008 ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/4c63cd36279b7e8448d09651a51ed8a6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VCR</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Virginia Coast Reserve</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Salt marsh creek</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Coastal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Upper Phillips Creek inundation experiment (1st)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Inundation; wrack (Juncus) manipulation</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Total plant biomass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1994-2013</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>16</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>knb-lter-vcr.168.24</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Christian, R. (2019). Data from: “End of Year Biomass for the 1st UPC Inundation Experiment in Upper Phillips Creek marsh 1999-2014 ver 24.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/3854929ce06dc8c667eff9615adb730f</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AND</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Andrews Forest</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Temperate conifer forest</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Forest</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TV010 experimental watersheds (WS06 clearcut, WS07 shelterwood, WS08 control)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Forest harvest (clearcut; shelterwood)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Tree diameter at breast height (cm)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2002-2014</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>knb-lter-and.2742.28</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Franklin, J. F., Bell, D. M., Remillard, S. M., Pabst, R. J., Bluhm, A. &amp; Powers, M. (2025). Data from: “Long-term growth, mortality and regeneration of trees in permanent vegetation plots in the Pacific Northwest, 1910 to present ver 28.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/dc4be3db15934e0e5eb4820f56e5d569</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HBR</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Hubbard Brook</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Northern hardwood forest</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Forest</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MELNHE (Multiple Element Limitation in Northern Hardwood Ecosystems)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Fertilization (N, P, Ca)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Litterfall mass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Flux</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2009-2021</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>13</v>
+      </c>
+      <c r="K9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>knb-lter-hbr.404.1</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Yanai, R. D., Fisk, M. C., Vadeboncoeur, M. A., Zukswert, J. M., Mann, T., Young, A., Walsh, G., Morley, M. &amp; See, C. R. (2024). Data from: “Multiple Element Limitation in Northern Hardwood Ecosystems (MELNHE): Litterfall mass 2009-2022 ver 1.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/e2d437bddf1166a733b0df09c87f89f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HFR</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Harvard Forest</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Temperate deciduous forest</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Forest</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Prospect Hill soil warming experiment</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Soil warming</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Soil respiration (CO2 flux)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Flux</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1991-2021</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>31</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>knb-lter-hfr.5.37</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Frey, S. &amp; Melillo, J. (2024). Data from: “Prospect Hill Soil Warming Experiment at Harvard Forest since 1991 ver 37.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/abf59a218a5868baf5b2c073a7dd1d7f</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LUQ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Luquillo</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Tropical wet forest</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Forest</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Canopy Trimming Experiment (CTE)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Canopy trimming; debris addition</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Soil CO2 flux</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Flux</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2003-2009</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>7</v>
+      </c>
+      <c r="K11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>knb-lter-luq.164.678951</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Silver, W. (2023). Data from: “Canopy Trimming Experiment (CTE) trace gases ver 678951.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/97823bf81da5abf22f8f9d8f3778fc58</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NTL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>North Temperate Lakes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Temperate lake</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Freshwater</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Cascade Project whole-lake nutrient addition</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Fertilization (N)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Chlorophyll (ug L-1; carbon proxy)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2011-2019</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>knb-lter-ntl.413.2</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Buelo, C. D., Pace, M. L., Carpenter, S. R., Stanley, E. H., Ortiz, D. A. &amp; Ha, D. T. (2022). Data from: “Cascade Project at North Temperate Lakes LTER – Daily Bloom Data for Whole Lake Experiments 2011 - 2019 ver 2.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5a9862187368b616bed8e20381343717</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CDR</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cedar Creek</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Prairie grassland</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Grassland</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BioCON</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CO2 enrichment; N fertilization; species richness</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Aboveground biomass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1998-2021</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>24</v>
+      </c>
+      <c r="K13" t="n">
+        <v>33</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>knb-lter-cdr.302.13</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Reich, P. (2024). Data from: “Plant aboveground biomass data: BioCON : Biodiversity, Elevated CO2, and N Enrichment ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/c153c4eb2414bb1ec2ab8b07adc17ef2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>KBS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Kellogg Biological Station</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cropland</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Grassland</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Main Cropping System Experiment (MCSE)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Cropping system / management intensity</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Aboveground net primary production (g m-2)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1990-2022</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>33</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>knb-lter-kbs.19.85</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Robertson, G. &amp; Snapp, S. (2020). Data from: “Annual Net Primary Production on the Main Cropping System Experiment at the Kellogg Biological Station, Hickory Corners, MI (1990 to 2018) ver 85.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f9b2a038b8a7ad43a252587a84935f30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KNZ</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Konza Prairie</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tallgrass prairie</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Grassland</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Belowground Plot Experiment (PBB01)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Fire; mowing; N and P fertilization</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Aboveground net primary production (g m-2)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>1986-2021</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>36</v>
+      </c>
+      <c r="K15" t="n">
+        <v>15</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>knb-lter-knz.57.15</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Blair, J. &amp; Zeglin, L. (2023). Data from: “PBB01 Belowground Plot Experiment: Aboveground net primary productivity of tallgrass prairie based on accumulated plant biomass ver 15.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/d769700c0e40751bfb8b4fb8c34dabb2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SEV</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sevilleta</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Desert grassland</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Grassland</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>NFert experiment</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Fertilization (N)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Aboveground biomass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2004-2023</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>20</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>knb-lter-sev.186.208431</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Baur, L., Collins, S., Muldavin, E., Rudgers, J. A. &amp; Pockman, W. T. (2024). Data from: “Nitrogen Fertilization Experiment (NFert): Seasonal Biomass and Seasonal and Annual NPP Data at the Sevilleta National Wildlife Refuge, New Mexico ver 208431.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/9468c8bcda68c0a05c06499ec51b1d55</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ARC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Arctic LTER</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Arctic tussock tundra</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tundra</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Toolik Lake moist acidic tussock tundra experiment</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Fertilization; warming; shading</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Aboveground biomass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>1982-2015</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>7</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>1 (4)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>knb-lter-arc.10004.8</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Shaver, G. (2017). Data from: “Above ground plant biomass in a mesic acidic tussock tundra experimental site from 1982 to 2015 Arctic LTER, Toolik Lake, Alaska. ver 8.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/c3ef07e6ed81c1fc33e9bc20aff07093</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BNZ</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bonanza Creek</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Boreal forest / permafrost tundra</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tundra</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CiPEHR (Carbon in Permafrost Experimental Heating Research)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Warming (soil and air)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Net ecosystem exchange</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Flux</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2009-2021</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>13</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>3 (6)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>knb-lter-bnz.481.23</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Rodenhizer, H. G., Mauritz, M., Taylor, M., Ledman, J., Natali, S. &amp; Schuur, E. (2022). Data from: “Eight Mile Lake Research Watershed, Carbon in Permafrost Experimental Heating Research (CiPEHR): Half-hourly growing season, chamber-based, CO2 flux data, 2009-2021 ver 23.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5ee6a71835606934afda8e3eb9a38763</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MCM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>McMurdo Dry Valleys</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Polar desert soil</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tundra</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Stoichiometry experiment (Bonney and Fryxell basins)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Nutrient addition (C, N, P)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Soil CO2 flux</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Flux</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2003-2010</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>knb-lter-mcm.4014.5</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Virginia, R. &amp; Wall, D. (2016). Data from: “McMurdo Dry Valleys Stoichiometry Experiment - CO2 ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f2c3854f11c24c54be3f3828c130746f</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NWT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Niwot Ridge</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Alpine tundra</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Tundra</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Snow x N x temperature experiment (Niwot Saddle)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Fertilization (N; ambient snow and temperature plots)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Aboveground biomass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2006-2019</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>13</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>knb-lter-nwt.13.7</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Suding, K. N., Smith, J. G. &amp; Ashton, I. W. (2024). Data from: “Increased temperature, N and snowpack experiment for north of saddle, 2006 - ongoing. ver 7.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/caacfd0b6e32b5a72f8fe3904ca897bf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Central Arizona-Phoenix</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sonoran Desert</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Desert Fertilization Experiment (CNdep)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Fertilization (N, P)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Aboveground biomass (g m-2)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Stock</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2008-2024</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>12</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>knb-lter-cap.632.17</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Grimm, N., Hall, S. J., Kaye, J. &amp; Allen, J. (2024). Data from: “Desert Fertilization Experiment: investigation of Sonoran desert ecosystem response to atmospheric deposition and experimental nutrient addition, ongoing since 2006 ver 17.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/fd7e336a9493e780777d97bb08ff2352</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Y86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -455,7 +1696,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table S1. Per-treatment statistics for the 83 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; tolerance 0.2), years to first detection of a significant trend (directional treatments only), the number, percentage (of consecutive measurement transitions), and years of sign flips, and the P-value and directional call when the trend analysis is repeated on the log response ratio.</t>
+          <t>Table S2. Per-treatment statistics for the 83 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; tolerance 0.2), years to first detection of a significant trend (directional treatments only), the number, percentage (of consecutive measurement transitions), and years of sign flips, and the P-value and directional call when the trend analysis is repeated on the log response ratio.</t>
         </is>
       </c>
     </row>
@@ -8864,7 +10105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8888,7 +10129,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table S2. SiZer results for the 79 treatment-experiment combinations with at least five timepoints: number of significant slope changes at a 5-year bandwidth, the years at which they occurred, and segment slopes with P-values.</t>
+          <t>Table S3. SiZer results for the 79 treatment-experiment combinations with at least five timepoints: number of significant slope changes at a 5-year bandwidth, the years at which they occurred, and segment slopes with P-values.</t>
         </is>
       </c>
     </row>
@@ -12330,1247 +13571,6 @@
       </c>
       <c r="J82" t="n">
         <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Table S3. Details of the 18 case-study datasets: setting, experiment, manipulation, response variable and type, years analyzed, number of years sampled, number of analyzable treatments (in parentheses, the number screened), EDI data-package identifier, and data citation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Site Name</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Setting</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Ecosystem Type</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Experiment</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Manipulation</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Response Variable</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Response Type</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Years Analyzed</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>N Years Sampled</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>N Treatments</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>EDI Package</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Data Citation</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>GCE</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Georgia Coastal Ecosystems</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Salt marsh</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Coastal</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Tidal marsh disturbance experiment (PLT-GCED-2207)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Vegetation removal (disturbance)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Vegetation cover (%; carbon proxy)</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Proxy</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2010-2020</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>11</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>knb-lter-gce.786.13</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Pennings, S. C. (2022). Data from: “Critical slowing down: vegetation height, cover and composition assess resilience of tidal fresh, brackish and salt marshes following experimental disturbance at twelve sites across the estuarine landscape ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/6df40a30859a7293db9a76fc4fff8cec</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>PIE</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Plum Island Ecosystems</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Salt marsh creek</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Coastal</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>TIDE nutrient-enrichment experiment</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Fertilization (NO3)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Plant shoot mass</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2004-2020</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>17</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>knb-lter-pie.202.5</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Deegan, L., Warren, S. &amp; Mozdzer, T. (2022). Data from: “Marsh plant species shoot height, weight and diameters for Rowley River tidal creeks associated with long term fertilization experiments, Rowley and Ipswich, MA. ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/226fb7db2c7b9f8119e40c937b1a19a0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>SBC</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Santa Barbara Coastal</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Kelp forest reef</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Coastal</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Long-term kelp removal experiment</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Vegetation removal (annual and continual kelp removal)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Algal dry biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2008-2023</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>knb-lter-sbc.119.13</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Reed, D. C. &amp; Miller, R. J. (2024). Data from: “SBC LTER: Reef: Long-term experiment: biomass of kelp forest species, ongoing since 2008 ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/4c63cd36279b7e8448d09651a51ed8a6</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>VCR</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Virginia Coast Reserve</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Salt marsh creek</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Coastal</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Upper Phillips Creek inundation experiment (1st)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Inundation; wrack (Juncus) manipulation</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Total plant biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>1994-2013</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>16</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>knb-lter-vcr.168.24</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Christian, R. (2019). Data from: “End of Year Biomass for the 1st UPC Inundation Experiment in Upper Phillips Creek marsh 1999-2014 ver 24.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/3854929ce06dc8c667eff9615adb730f</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AND</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Andrews Forest</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Temperate conifer forest</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>TV010 experimental watersheds (WS06 clearcut, WS07 shelterwood, WS08 control)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Forest harvest (clearcut; shelterwood)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Tree diameter at breast height (cm)</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2002-2014</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>3</v>
-      </c>
-      <c r="K8" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>knb-lter-and.2742.28</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Franklin, J. F., Bell, D. M., Remillard, S. M., Pabst, R. J., Bluhm, A. &amp; Powers, M. (2025). Data from: “Long-term growth, mortality and regeneration of trees in permanent vegetation plots in the Pacific Northwest, 1910 to present ver 28.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/dc4be3db15934e0e5eb4820f56e5d569</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>HBR</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Hubbard Brook</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Northern hardwood forest</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>MELNHE (Multiple Element Limitation in Northern Hardwood Ecosystems)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Fertilization (N, P, Ca)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Litterfall mass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Flux</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2009-2021</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>13</v>
-      </c>
-      <c r="K9" t="n">
-        <v>4</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>knb-lter-hbr.404.1</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Yanai, R. D., Fisk, M. C., Vadeboncoeur, M. A., Zukswert, J. M., Mann, T., Young, A., Walsh, G., Morley, M. &amp; See, C. R. (2024). Data from: “Multiple Element Limitation in Northern Hardwood Ecosystems (MELNHE): Litterfall mass 2009-2022 ver 1.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/e2d437bddf1166a733b0df09c87f89f1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>HFR</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Harvard Forest</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Temperate deciduous forest</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Prospect Hill soil warming experiment</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Soil warming</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Soil respiration (CO2 flux)</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Flux</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>1991-2021</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>31</v>
-      </c>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>knb-lter-hfr.5.37</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Frey, S. &amp; Melillo, J. (2024). Data from: “Prospect Hill Soil Warming Experiment at Harvard Forest since 1991 ver 37.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/abf59a218a5868baf5b2c073a7dd1d7f</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LUQ</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Luquillo</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Tropical wet forest</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Canopy Trimming Experiment (CTE)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Canopy trimming; debris addition</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Soil CO2 flux</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Flux</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2003-2009</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>7</v>
-      </c>
-      <c r="K11" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>knb-lter-luq.164.678951</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Silver, W. (2023). Data from: “Canopy Trimming Experiment (CTE) trace gases ver 678951.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/97823bf81da5abf22f8f9d8f3778fc58</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>NTL</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>North Temperate Lakes</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Temperate lake</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Freshwater</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Cascade Project whole-lake nutrient addition</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Fertilization (N)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Chlorophyll (ug L-1; carbon proxy)</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Proxy</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2011-2019</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>7</v>
-      </c>
-      <c r="K12" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>knb-lter-ntl.413.2</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Buelo, C. D., Pace, M. L., Carpenter, S. R., Stanley, E. H., Ortiz, D. A. &amp; Ha, D. T. (2022). Data from: “Cascade Project at North Temperate Lakes LTER – Daily Bloom Data for Whole Lake Experiments 2011 - 2019 ver 2.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5a9862187368b616bed8e20381343717</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CDR</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Cedar Creek</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Prairie grassland</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Grassland</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>BioCON</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>CO2 enrichment; N fertilization; species richness</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Aboveground biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>1998-2021</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>24</v>
-      </c>
-      <c r="K13" t="n">
-        <v>33</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>knb-lter-cdr.302.13</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Reich, P. (2024). Data from: “Plant aboveground biomass data: BioCON : Biodiversity, Elevated CO2, and N Enrichment ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/c153c4eb2414bb1ec2ab8b07adc17ef2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>KBS</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Kellogg Biological Station</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Cropland</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Grassland</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Main Cropping System Experiment (MCSE)</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Cropping system / management intensity</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Aboveground net primary production (g m-2)</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>1990-2022</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>33</v>
-      </c>
-      <c r="K14" t="n">
-        <v>5</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>knb-lter-kbs.19.85</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Robertson, G. &amp; Snapp, S. (2020). Data from: “Annual Net Primary Production on the Main Cropping System Experiment at the Kellogg Biological Station, Hickory Corners, MI (1990 to 2018) ver 85.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f9b2a038b8a7ad43a252587a84935f30</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>KNZ</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Konza Prairie</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Tallgrass prairie</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Grassland</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Belowground Plot Experiment (PBB01)</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Fire; mowing; N and P fertilization</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Aboveground net primary production (g m-2)</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>1986-2021</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>36</v>
-      </c>
-      <c r="K15" t="n">
-        <v>15</v>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>knb-lter-knz.57.15</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Blair, J. &amp; Zeglin, L. (2023). Data from: “PBB01 Belowground Plot Experiment: Aboveground net primary productivity of tallgrass prairie based on accumulated plant biomass ver 15.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/d769700c0e40751bfb8b4fb8c34dabb2</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SEV</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Sevilleta</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Desert grassland</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Grassland</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>NFert experiment</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Fertilization (N)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Aboveground biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>2004-2023</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>20</v>
-      </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>knb-lter-sev.186.208431</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Baur, L., Collins, S., Muldavin, E., Rudgers, J. A. &amp; Pockman, W. T. (2024). Data from: “Nitrogen Fertilization Experiment (NFert): Seasonal Biomass and Seasonal and Annual NPP Data at the Sevilleta National Wildlife Refuge, New Mexico ver 208431.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/9468c8bcda68c0a05c06499ec51b1d55</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>ARC</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Arctic LTER</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Arctic tussock tundra</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Tundra</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Toolik Lake moist acidic tussock tundra experiment</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Fertilization; warming; shading</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Aboveground biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>1982-2015</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>7</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>1 (4)</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>knb-lter-arc.10004.8</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Shaver, G. (2017). Data from: “Above ground plant biomass in a mesic acidic tussock tundra experimental site from 1982 to 2015 Arctic LTER, Toolik Lake, Alaska. ver 8.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/c3ef07e6ed81c1fc33e9bc20aff07093</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>BNZ</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Bonanza Creek</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Boreal forest / permafrost tundra</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Tundra</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>CiPEHR (Carbon in Permafrost Experimental Heating Research)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Warming (soil and air)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Net ecosystem exchange</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Flux</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2009-2021</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>13</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>3 (6)</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>knb-lter-bnz.481.23</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Rodenhizer, H. G., Mauritz, M., Taylor, M., Ledman, J., Natali, S. &amp; Schuur, E. (2022). Data from: “Eight Mile Lake Research Watershed, Carbon in Permafrost Experimental Heating Research (CiPEHR): Half-hourly growing season, chamber-based, CO2 flux data, 2009-2021 ver 23.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5ee6a71835606934afda8e3eb9a38763</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>MCM</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>McMurdo Dry Valleys</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Polar desert soil</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Tundra</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Stoichiometry experiment (Bonney and Fryxell basins)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Nutrient addition (C, N, P)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Soil CO2 flux</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Flux</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2003-2010</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>5</v>
-      </c>
-      <c r="K19" t="n">
-        <v>5</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>knb-lter-mcm.4014.5</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Virginia, R. &amp; Wall, D. (2016). Data from: “McMurdo Dry Valleys Stoichiometry Experiment - CO2 ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f2c3854f11c24c54be3f3828c130746f</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>NWT</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Niwot Ridge</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Alpine tundra</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Tundra</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Snow x N x temperature experiment (Niwot Saddle)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Fertilization (N; ambient snow and temperature plots)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Aboveground biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>2006-2019</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>13</v>
-      </c>
-      <c r="K20" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>knb-lter-nwt.13.7</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Suding, K. N., Smith, J. G. &amp; Ashton, I. W. (2024). Data from: “Increased temperature, N and snowpack experiment for north of saddle, 2006 - ongoing. ver 7.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/caacfd0b6e32b5a72f8fe3904ca897bf</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>CAP</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Central Arizona-Phoenix</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Sonoran Desert</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Urban</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Desert Fertilization Experiment (CNdep)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Fertilization (N, P)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Aboveground biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2008-2024</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>12</v>
-      </c>
-      <c r="K21" t="n">
-        <v>3</v>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>knb-lter-cap.632.17</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Grimm, N., Hall, S. J., Kaye, J. &amp; Allen, J. (2024). Data from: “Desert Fertilization Experiment: investigation of Sonoran desert ecosystem response to atmospheric deposition and experimental nutrient addition, ongoing since 2006 ver 17.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/fd7e336a9493e780777d97bb08ff2352</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
GCE and SBC: download from EDI reproducibly; fix SBC missing-value code
- registry now records the EDI entity IDs for knb-lter-gce.786.13 and
  knb-lter-sbc.119.13; both raw files are downloaded, checksummed and
  manifested like the other 16 datasets
- download_from_edi() falls back to EDI's DataONE member node when
  PASTA refuses anonymous API requests
- preprocess_gce reads the EDI entity layout; the regenerated ready file
  is identical to the hand-processed one (revision confirmed)
- preprocess_sbc converts the -99999 missing-value code to NA before
  summing. The hand-processed file had summed the code into 11
  transect-month biomass totals (~ -99,000 g m-2), which removed 2008
  from the record and inflated the CV of the continual-removal
  treatment; it also lacked 14 November-2014 transect surveys
- downstream outputs regenerated: trend classes unchanged; sign flips
  54 of 83 (65%); tolerance-0.1 sensitivity 55%

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -9740,31 +9740,31 @@
         <v>0</v>
       </c>
       <c r="I83" t="n">
-        <v>0.4986</v>
+        <v>0.1545</v>
       </c>
       <c r="J83" t="n">
-        <v>0.0359</v>
+        <v>0.1393</v>
       </c>
       <c r="K83" t="n">
-        <v>0.1821</v>
+        <v>0.2121</v>
       </c>
       <c r="L83" t="n">
-        <v>0.7218</v>
+        <v>0.741</v>
       </c>
       <c r="M83" t="n">
+        <v>16</v>
+      </c>
+      <c r="N83" t="n">
         <v>15</v>
       </c>
-      <c r="N83" t="n">
-        <v>14</v>
-      </c>
       <c r="O83" t="n">
-        <v>-0.3581</v>
+        <v>-0.2086</v>
       </c>
       <c r="P83" t="n">
-        <v>-0.3414</v>
+        <v>-0.32</v>
       </c>
       <c r="Q83" t="n">
-        <v>0.0167</v>
+        <v>-0.1113</v>
       </c>
       <c r="R83" t="inlineStr">
         <is>
@@ -9782,18 +9782,16 @@
         </is>
       </c>
       <c r="U83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V83" t="n">
-        <v>0</v>
-      </c>
-      <c r="W83" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>6.6667</v>
+      </c>
+      <c r="W83" t="n">
+        <v>2009</v>
       </c>
       <c r="X83" t="n">
-        <v>0.6223</v>
+        <v>0.2371</v>
       </c>
       <c r="Y83" t="inlineStr">
         <is>
@@ -9838,19 +9836,19 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>0.0001</v>
+        <v>-0.0001</v>
       </c>
       <c r="I84" t="n">
-        <v>0.6748</v>
+        <v>0.4091</v>
       </c>
       <c r="J84" t="n">
-        <v>0.0152</v>
+        <v>0.0575</v>
       </c>
       <c r="K84" t="n">
-        <v>1.0351</v>
+        <v>0.4797</v>
       </c>
       <c r="L84" t="n">
-        <v>1.0399</v>
+        <v>1.1561</v>
       </c>
       <c r="M84" t="n">
         <v>14</v>
@@ -9859,13 +9857,13 @@
         <v>13</v>
       </c>
       <c r="O84" t="n">
-        <v>0.0626</v>
+        <v>0.0643</v>
       </c>
       <c r="P84" t="n">
-        <v>0.1008</v>
+        <v>0.0853</v>
       </c>
       <c r="Q84" t="n">
-        <v>0.0382</v>
+        <v>0.021</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
@@ -9874,25 +9872,27 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T84" t="n">
-        <v>4</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U84" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V84" t="n">
-        <v>30.7692</v>
+        <v>38.4615</v>
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>2012; 2015; 2018; 2020</t>
+          <t>2011; 2012; 2015; 2018; 2020</t>
         </is>
       </c>
       <c r="X84" t="n">
-        <v>0.3646</v>
+        <v>0.3272</v>
       </c>
       <c r="Y84" t="inlineStr">
         <is>
@@ -13425,7 +13425,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F79" t="n">
         <v>0</v>
@@ -13436,10 +13436,10 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>-0.005572</v>
+        <v>-0.01232</v>
       </c>
       <c r="I79" t="n">
-        <v>0.4986</v>
+        <v>0.1545</v>
       </c>
       <c r="J79" t="n">
         <v>5</v>
@@ -13478,10 +13478,10 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>0.031698</v>
+        <v>-0.031785</v>
       </c>
       <c r="I80" t="n">
-        <v>0.6748</v>
+        <v>0.4091</v>
       </c>
       <c r="J80" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
Correct legacy processing choices in KBS, ARC, CDR and AND
KBS  source is EDI revision 85 (1990-2018, as cited); whole-plant biomass
     uses the WHOLE fraction where reported instead of summing WHOLE with
     its own components (legacy totals were ~2x), LITTER excluded
ARC  late-July harvest only (the two July-1983 harvests were summed),
     aboveground categories only (belowground and litter were included in
     some years), all harvested quadrats, 2015 recovered from raw masses
CDR  litter and bare-ground records excluded from aboveground biomass;
     August peak harvest only (June harvests exist only for 1998-2011)
AND  all live stems (status 1-3); status-1-only dropped ingrowth

Downstream outputs regenerated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -1187,11 +1187,11 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1990-2022</t>
+          <t>1990-2018</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="K14" t="n">
         <v>5</v>
@@ -2127,16 +2127,16 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0143</v>
+        <v>0.0032</v>
       </c>
       <c r="J4" t="n">
-        <v>0.9995000000000001</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1597</v>
+        <v>0.18</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5082</v>
+        <v>0.5184</v>
       </c>
       <c r="M4" t="n">
         <v>3</v>
@@ -2145,13 +2145,13 @@
         <v>12</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.8532999999999999</v>
+        <v>-0.8548</v>
       </c>
       <c r="P4" t="n">
-        <v>-0.6855</v>
+        <v>-0.668</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.1678</v>
+        <v>0.1868</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
         </is>
       </c>
       <c r="X4" t="n">
-        <v>0.0436</v>
+        <v>0.03</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
@@ -2226,16 +2226,16 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0447</v>
+        <v>0.0052</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9951</v>
+        <v>0.9999</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2089</v>
+        <v>0.2221</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4614</v>
+        <v>0.4633</v>
       </c>
       <c r="M5" t="n">
         <v>3</v>
@@ -2244,13 +2244,13 @@
         <v>12</v>
       </c>
       <c r="O5" t="n">
-        <v>-1.0177</v>
+        <v>-1.0192</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.7885</v>
+        <v>-0.7863</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.2292</v>
+        <v>0.2329</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -2277,11 +2277,11 @@
         </is>
       </c>
       <c r="X5" t="n">
-        <v>0.082</v>
+        <v>0.036</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>non-directional</t>
+          <t>increasing</t>
         </is>
       </c>
     </row>
@@ -2322,34 +2322,34 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2979</v>
+        <v>0.1816</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3447</v>
+        <v>0.3946</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2361</v>
+        <v>0.2404</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3925</v>
+        <v>1.4524</v>
       </c>
       <c r="M6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N6" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="O6" t="n">
-        <v>0.2336</v>
+        <v>0.3073</v>
       </c>
       <c r="P6" t="n">
-        <v>0.31</v>
+        <v>0.3492</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.0419</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -2378,7 +2378,7 @@
         </is>
       </c>
       <c r="X6" t="n">
-        <v>0.3015</v>
+        <v>0.2228</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -3024,16 +3024,16 @@
         <v>0.0001</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3906</v>
+        <v>0.445</v>
       </c>
       <c r="J13" t="n">
-        <v>0.062</v>
+        <v>0.0494</v>
       </c>
       <c r="K13" t="n">
-        <v>0.3957</v>
+        <v>0.4749</v>
       </c>
       <c r="L13" t="n">
-        <v>1.5842</v>
+        <v>1.5724</v>
       </c>
       <c r="M13" t="n">
         <v>14</v>
@@ -3042,13 +3042,13 @@
         <v>14</v>
       </c>
       <c r="O13" t="n">
-        <v>0.2921</v>
+        <v>0.2701</v>
       </c>
       <c r="P13" t="n">
-        <v>0.3925</v>
+        <v>0.3636</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.1004</v>
+        <v>0.0935</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -3057,25 +3057,27 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T13" t="n">
-        <v>12</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V13" t="n">
-        <v>46.1538</v>
+        <v>30.7692</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>2013; 2014; 2015; 2016; 2020; 2021</t>
+          <t>2015; 2016; 2020; 2021</t>
         </is>
       </c>
       <c r="X13" t="n">
-        <v>0.5968</v>
+        <v>0.6729000000000001</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
@@ -3123,16 +3125,16 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>0.9657</v>
+        <v>0.9769</v>
       </c>
       <c r="J14" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="K14" t="n">
-        <v>0.239</v>
+        <v>0.237</v>
       </c>
       <c r="L14" t="n">
-        <v>1.7166</v>
+        <v>1.8432</v>
       </c>
       <c r="M14" t="n">
         <v>10</v>
@@ -3141,13 +3143,13 @@
         <v>9</v>
       </c>
       <c r="O14" t="n">
-        <v>0.4373</v>
+        <v>0.5133</v>
       </c>
       <c r="P14" t="n">
-        <v>0.5165999999999999</v>
+        <v>0.5877</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.0793</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -3176,7 +3178,7 @@
         </is>
       </c>
       <c r="X14" t="n">
-        <v>0.8399</v>
+        <v>0.8234</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
@@ -3224,16 +3226,16 @@
         <v>-0.0002</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3295</v>
+        <v>0.1855</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1187</v>
+        <v>0.2078</v>
       </c>
       <c r="K15" t="n">
-        <v>0.3578</v>
+        <v>0.328</v>
       </c>
       <c r="L15" t="n">
-        <v>1.6268</v>
+        <v>1.6982</v>
       </c>
       <c r="M15" t="n">
         <v>10</v>
@@ -3242,13 +3244,13 @@
         <v>9</v>
       </c>
       <c r="O15" t="n">
-        <v>0.6341</v>
+        <v>0.7332</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4309</v>
+        <v>0.4837</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.2032</v>
+        <v>-0.2494</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -3266,18 +3268,18 @@
         </is>
       </c>
       <c r="U15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>22.2222</v>
+        <v>0</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>2020; 2021</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="X15" t="n">
-        <v>0.2925</v>
+        <v>0.1372</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
@@ -3322,19 +3324,19 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="I16" t="n">
-        <v>0.8132</v>
+        <v>0.3104</v>
       </c>
       <c r="J16" t="n">
-        <v>0.0217</v>
+        <v>0.3307</v>
       </c>
       <c r="K16" t="n">
-        <v>0.1096</v>
+        <v>0.1236</v>
       </c>
       <c r="L16" t="n">
-        <v>1.3575</v>
+        <v>1.2864</v>
       </c>
       <c r="M16" t="n">
         <v>5</v>
@@ -3343,13 +3345,13 @@
         <v>4</v>
       </c>
       <c r="O16" t="n">
-        <v>0.2942</v>
+        <v>0.172</v>
       </c>
       <c r="P16" t="n">
-        <v>0.3009</v>
+        <v>0.2455</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.0067</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -3378,7 +3380,7 @@
         </is>
       </c>
       <c r="X16" t="n">
-        <v>0.7542</v>
+        <v>0.3548</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
@@ -3419,23 +3421,23 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H17" t="n">
         <v>-0.0001</v>
       </c>
       <c r="I17" t="n">
-        <v>0.7228</v>
+        <v>0.5383</v>
       </c>
       <c r="J17" t="n">
-        <v>0.0191</v>
+        <v>0.0564</v>
       </c>
       <c r="K17" t="n">
-        <v>0.3221</v>
+        <v>0.2996</v>
       </c>
       <c r="L17" t="n">
-        <v>1.2949</v>
+        <v>1.2659</v>
       </c>
       <c r="M17" t="n">
         <v>9</v>
@@ -3444,13 +3446,13 @@
         <v>9</v>
       </c>
       <c r="O17" t="n">
-        <v>0.2565</v>
+        <v>0.2638</v>
       </c>
       <c r="P17" t="n">
-        <v>0.2034</v>
+        <v>0.187</v>
       </c>
       <c r="Q17" t="n">
-        <v>-0.0531</v>
+        <v>-0.07679999999999999</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -3479,7 +3481,7 @@
         </is>
       </c>
       <c r="X17" t="n">
-        <v>0.4578</v>
+        <v>0.3699</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
@@ -3524,19 +3526,19 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>-0.0001</v>
       </c>
       <c r="I18" t="n">
-        <v>0.8443000000000001</v>
+        <v>0.6276</v>
       </c>
       <c r="J18" t="n">
-        <v>0.0059</v>
+        <v>0.0354</v>
       </c>
       <c r="K18" t="n">
-        <v>0.2679</v>
+        <v>0.2935</v>
       </c>
       <c r="L18" t="n">
-        <v>1.4781</v>
+        <v>1.4794</v>
       </c>
       <c r="M18" t="n">
         <v>9</v>
@@ -3545,13 +3547,13 @@
         <v>9</v>
       </c>
       <c r="O18" t="n">
-        <v>0.469</v>
+        <v>0.5152</v>
       </c>
       <c r="P18" t="n">
-        <v>0.3607</v>
+        <v>0.3534</v>
       </c>
       <c r="Q18" t="n">
-        <v>-0.1083</v>
+        <v>-0.1618</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -3569,18 +3571,18 @@
         </is>
       </c>
       <c r="U18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V18" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>2015; 2016</t>
         </is>
       </c>
       <c r="X18" t="n">
-        <v>0.8691</v>
+        <v>0.6697</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
@@ -3625,19 +3627,19 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>-0.0005</v>
+        <v>-0.0007</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0156</v>
+        <v>0.0064</v>
       </c>
       <c r="J19" t="n">
-        <v>0.5904</v>
+        <v>0.6784</v>
       </c>
       <c r="K19" t="n">
-        <v>0.322</v>
+        <v>0.3551</v>
       </c>
       <c r="L19" t="n">
-        <v>2.1531</v>
+        <v>2.4814</v>
       </c>
       <c r="M19" t="n">
         <v>9</v>
@@ -3646,13 +3648,13 @@
         <v>8</v>
       </c>
       <c r="O19" t="n">
-        <v>0.9641999999999999</v>
+        <v>1.1711</v>
       </c>
       <c r="P19" t="n">
-        <v>0.7193000000000001</v>
+        <v>0.8501</v>
       </c>
       <c r="Q19" t="n">
-        <v>-0.2449</v>
+        <v>-0.321</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -3679,7 +3681,7 @@
         </is>
       </c>
       <c r="X19" t="n">
-        <v>0.0089</v>
+        <v>0.0047</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -3720,23 +3722,23 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H20" t="n">
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>0.0038</v>
+        <v>0.5589</v>
       </c>
       <c r="J20" t="n">
-        <v>0.3355</v>
+        <v>0.0165</v>
       </c>
       <c r="K20" t="n">
-        <v>0.159</v>
+        <v>0.1963</v>
       </c>
       <c r="L20" t="n">
-        <v>1.091</v>
+        <v>1.0363</v>
       </c>
       <c r="M20" t="n">
         <v>23</v>
@@ -3745,13 +3747,13 @@
         <v>23</v>
       </c>
       <c r="O20" t="n">
-        <v>-0.0571</v>
+        <v>-0.0921</v>
       </c>
       <c r="P20" t="n">
-        <v>0.0747</v>
+        <v>0.0172</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.1319</v>
+        <v>0.1093</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -3764,25 +3766,25 @@
         </is>
       </c>
       <c r="T20" t="n">
-        <v>3.0007</v>
+        <v>11.0007</v>
       </c>
       <c r="U20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="V20" t="n">
-        <v>18.1818</v>
+        <v>40.9091</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>1999; 2004; 2005; 2007</t>
+          <t>1999; 2003; 2005; 2006; 2010; 2011; 2015; 2016; 2017</t>
         </is>
       </c>
       <c r="X20" t="n">
-        <v>0.0031</v>
+        <v>0.4577</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
@@ -3819,23 +3821,23 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>decreasing</t>
         </is>
       </c>
       <c r="H21" t="n">
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0222</v>
       </c>
       <c r="J21" t="n">
-        <v>0.1347</v>
+        <v>0.2157</v>
       </c>
       <c r="K21" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.0997</v>
       </c>
       <c r="L21" t="n">
-        <v>1.1268</v>
+        <v>1.161</v>
       </c>
       <c r="M21" t="n">
         <v>24</v>
@@ -3844,13 +3846,13 @@
         <v>23</v>
       </c>
       <c r="O21" t="n">
-        <v>0.1884</v>
+        <v>0.2839</v>
       </c>
       <c r="P21" t="n">
-        <v>0.1162</v>
+        <v>0.1446</v>
       </c>
       <c r="Q21" t="n">
-        <v>-0.0722</v>
+        <v>-0.1393</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -3859,31 +3861,29 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>5.9986</v>
       </c>
       <c r="U21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V21" t="n">
-        <v>17.3913</v>
+        <v>8.6957</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>2009; 2010; 2020; 2021</t>
+          <t>2020; 2021</t>
         </is>
       </c>
       <c r="X21" t="n">
-        <v>0.0733</v>
+        <v>0.0198</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>non-directional</t>
+          <t>decreasing</t>
         </is>
       </c>
     </row>
@@ -3924,19 +3924,19 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>-0.0001</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0.4005</v>
+        <v>0.6807</v>
       </c>
       <c r="J22" t="n">
-        <v>0.0595</v>
+        <v>0.0146</v>
       </c>
       <c r="K22" t="n">
-        <v>0.4173</v>
+        <v>0.4627</v>
       </c>
       <c r="L22" t="n">
-        <v>1.4556</v>
+        <v>1.437</v>
       </c>
       <c r="M22" t="n">
         <v>14</v>
@@ -3945,13 +3945,13 @@
         <v>14</v>
       </c>
       <c r="O22" t="n">
-        <v>0.5405</v>
+        <v>0.5503</v>
       </c>
       <c r="P22" t="n">
-        <v>0.2713</v>
+        <v>0.2383</v>
       </c>
       <c r="Q22" t="n">
-        <v>-0.2692</v>
+        <v>-0.3119</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -3964,7 +3964,7 @@
         </is>
       </c>
       <c r="T22" t="n">
-        <v>10.0014</v>
+        <v>8.9993</v>
       </c>
       <c r="U22" t="n">
         <v>2</v>
@@ -3978,7 +3978,7 @@
         </is>
       </c>
       <c r="X22" t="n">
-        <v>0.2823</v>
+        <v>0.4647</v>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
@@ -4026,16 +4026,16 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>0.8794</v>
+        <v>0.7953</v>
       </c>
       <c r="J23" t="n">
-        <v>0.0031</v>
+        <v>0.0089</v>
       </c>
       <c r="K23" t="n">
-        <v>0.2239</v>
+        <v>0.2741</v>
       </c>
       <c r="L23" t="n">
-        <v>1.1248</v>
+        <v>1.0702</v>
       </c>
       <c r="M23" t="n">
         <v>10</v>
@@ -4044,13 +4044,13 @@
         <v>9</v>
       </c>
       <c r="O23" t="n">
-        <v>-0.06660000000000001</v>
+        <v>-0.0882</v>
       </c>
       <c r="P23" t="n">
-        <v>0.094</v>
+        <v>0.03</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.1606</v>
+        <v>0.1182</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -4063,7 +4063,7 @@
         </is>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
+        <v>3.0007</v>
       </c>
       <c r="U23" t="n">
         <v>2</v>
@@ -4077,7 +4077,7 @@
         </is>
       </c>
       <c r="X23" t="n">
-        <v>0.9277</v>
+        <v>0.7073</v>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
@@ -4125,16 +4125,16 @@
         <v>-0.0001</v>
       </c>
       <c r="I24" t="n">
-        <v>0.7306</v>
+        <v>0.7068</v>
       </c>
       <c r="J24" t="n">
-        <v>0.0156</v>
+        <v>0.0187</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2301</v>
+        <v>0.2477</v>
       </c>
       <c r="L24" t="n">
-        <v>2.0807</v>
+        <v>2.3198</v>
       </c>
       <c r="M24" t="n">
         <v>10</v>
@@ -4143,13 +4143,13 @@
         <v>9</v>
       </c>
       <c r="O24" t="n">
-        <v>0.7301</v>
+        <v>0.8411</v>
       </c>
       <c r="P24" t="n">
-        <v>0.7095</v>
+        <v>0.8156</v>
       </c>
       <c r="Q24" t="n">
-        <v>-0.0206</v>
+        <v>-0.0255</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -4178,7 +4178,7 @@
         </is>
       </c>
       <c r="X24" t="n">
-        <v>0.8292</v>
+        <v>0.8295</v>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
@@ -4223,19 +4223,19 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0.6388</v>
+        <v>0.9639</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0828</v>
+        <v>0.0008</v>
       </c>
       <c r="K25" t="n">
-        <v>0.1338</v>
+        <v>0.1645</v>
       </c>
       <c r="L25" t="n">
-        <v>1.3842</v>
+        <v>1.2848</v>
       </c>
       <c r="M25" t="n">
         <v>5</v>
@@ -4244,13 +4244,13 @@
         <v>4</v>
       </c>
       <c r="O25" t="n">
-        <v>0.3082</v>
+        <v>0.2813</v>
       </c>
       <c r="P25" t="n">
-        <v>0.3181</v>
+        <v>0.2385</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.009900000000000001</v>
+        <v>-0.0428</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -4268,18 +4268,18 @@
         </is>
       </c>
       <c r="U25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>2010; 2011</t>
         </is>
       </c>
       <c r="X25" t="n">
-        <v>0.6636</v>
+        <v>0.9524</v>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
@@ -4327,16 +4327,16 @@
         <v>-0.0001</v>
       </c>
       <c r="I26" t="n">
-        <v>0.3694</v>
+        <v>0.4761</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1162</v>
+        <v>0.07489999999999999</v>
       </c>
       <c r="K26" t="n">
-        <v>0.2548</v>
+        <v>0.2713</v>
       </c>
       <c r="L26" t="n">
-        <v>1.1496</v>
+        <v>1.1506</v>
       </c>
       <c r="M26" t="n">
         <v>9</v>
@@ -4345,13 +4345,13 @@
         <v>9</v>
       </c>
       <c r="O26" t="n">
-        <v>0.244</v>
+        <v>0.1795</v>
       </c>
       <c r="P26" t="n">
-        <v>0.107</v>
+        <v>0.1064</v>
       </c>
       <c r="Q26" t="n">
-        <v>-0.137</v>
+        <v>-0.0731</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
@@ -4360,27 +4360,25 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T26" t="n">
+        <v>3.0007</v>
       </c>
       <c r="U26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V26" t="n">
-        <v>37.5</v>
+        <v>62.5</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2015; 2016; 2021</t>
+          <t>2015; 2016; 2018; 2019; 2021</t>
         </is>
       </c>
       <c r="X26" t="n">
-        <v>0.411</v>
+        <v>0.4472</v>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
@@ -4428,16 +4426,16 @@
         <v>0.0001</v>
       </c>
       <c r="I27" t="n">
-        <v>0.5167</v>
+        <v>0.6738</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0624</v>
+        <v>0.0268</v>
       </c>
       <c r="K27" t="n">
-        <v>0.2201</v>
+        <v>0.1988</v>
       </c>
       <c r="L27" t="n">
-        <v>1.651</v>
+        <v>1.7873</v>
       </c>
       <c r="M27" t="n">
         <v>9</v>
@@ -4446,13 +4444,13 @@
         <v>9</v>
       </c>
       <c r="O27" t="n">
-        <v>0.4479</v>
+        <v>0.5608</v>
       </c>
       <c r="P27" t="n">
-        <v>0.4776</v>
+        <v>0.5624</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.0296</v>
+        <v>0.0016</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
@@ -4481,7 +4479,7 @@
         </is>
       </c>
       <c r="X27" t="n">
-        <v>0.6061</v>
+        <v>0.7813</v>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
@@ -4529,16 +4527,16 @@
         <v>0.0001</v>
       </c>
       <c r="I28" t="n">
-        <v>0.468</v>
+        <v>0.7028</v>
       </c>
       <c r="J28" t="n">
-        <v>0.0776</v>
+        <v>0.0221</v>
       </c>
       <c r="K28" t="n">
-        <v>0.3106</v>
+        <v>0.3569</v>
       </c>
       <c r="L28" t="n">
-        <v>1.0959</v>
+        <v>1.1595</v>
       </c>
       <c r="M28" t="n">
         <v>9</v>
@@ -4547,13 +4545,13 @@
         <v>8</v>
       </c>
       <c r="O28" t="n">
-        <v>-0.0163</v>
+        <v>0.1055</v>
       </c>
       <c r="P28" t="n">
-        <v>0.0486</v>
+        <v>0.0985</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.065</v>
+        <v>-0.007</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -4582,7 +4580,7 @@
         </is>
       </c>
       <c r="X28" t="n">
-        <v>0.549</v>
+        <v>0.6818</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
@@ -4630,16 +4628,16 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>0.4843</v>
+        <v>0.614</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0236</v>
+        <v>0.0123</v>
       </c>
       <c r="K29" t="n">
-        <v>0.1489</v>
+        <v>0.1803</v>
       </c>
       <c r="L29" t="n">
-        <v>1.2752</v>
+        <v>1.3144</v>
       </c>
       <c r="M29" t="n">
         <v>23</v>
@@ -4648,13 +4646,13 @@
         <v>23</v>
       </c>
       <c r="O29" t="n">
-        <v>0.2403</v>
+        <v>0.303</v>
       </c>
       <c r="P29" t="n">
-        <v>0.2332</v>
+        <v>0.2584</v>
       </c>
       <c r="Q29" t="n">
-        <v>-0.0071</v>
+        <v>-0.0446</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -4667,7 +4665,7 @@
         </is>
       </c>
       <c r="T29" t="n">
-        <v>1.9986</v>
+        <v>8</v>
       </c>
       <c r="U29" t="n">
         <v>1</v>
@@ -4679,7 +4677,7 @@
         <v>2021</v>
       </c>
       <c r="X29" t="n">
-        <v>0.6411</v>
+        <v>0.3923</v>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
@@ -4727,16 +4725,16 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>0.542</v>
+        <v>0.3207</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0171</v>
+        <v>0.0448</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1049</v>
+        <v>0.1088</v>
       </c>
       <c r="L30" t="n">
-        <v>1.0949</v>
+        <v>1.1288</v>
       </c>
       <c r="M30" t="n">
         <v>24</v>
@@ -4745,13 +4743,13 @@
         <v>23</v>
       </c>
       <c r="O30" t="n">
-        <v>0.0847</v>
+        <v>0.188</v>
       </c>
       <c r="P30" t="n">
-        <v>0.0851</v>
+        <v>0.1152</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.0004</v>
+        <v>-0.0728</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -4769,18 +4767,18 @@
         </is>
       </c>
       <c r="U30" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="V30" t="n">
-        <v>39.1304</v>
+        <v>17.3913</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>1999; 2009; 2011; 2012; 2014; 2015; 2016; 2020; 2021</t>
+          <t>2010; 2011; 2020; 2021</t>
         </is>
       </c>
       <c r="X30" t="n">
-        <v>0.4839</v>
+        <v>0.3001</v>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
@@ -4821,23 +4819,23 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>decreasing</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>-0.0005</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0035</v>
+        <v>0.094</v>
       </c>
       <c r="J31" t="n">
-        <v>0.9597</v>
+        <v>0.6615</v>
       </c>
       <c r="K31" t="n">
-        <v>0.1876</v>
+        <v>0.232</v>
       </c>
       <c r="L31" t="n">
-        <v>1.6738</v>
+        <v>1.8224</v>
       </c>
       <c r="M31" t="n">
         <v>5</v>
@@ -4846,13 +4844,13 @@
         <v>4</v>
       </c>
       <c r="O31" t="n">
-        <v>0.6074000000000001</v>
+        <v>0.7048</v>
       </c>
       <c r="P31" t="n">
-        <v>0.5014</v>
+        <v>0.5782</v>
       </c>
       <c r="Q31" t="n">
-        <v>-0.106</v>
+        <v>-0.1266</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
@@ -4861,11 +4859,13 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T31" t="n">
-        <v>3.0007</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U31" t="n">
         <v>0</v>
@@ -4879,11 +4879,11 @@
         </is>
       </c>
       <c r="X31" t="n">
-        <v>0.0013</v>
+        <v>0.0906</v>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>decreasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
@@ -4927,16 +4927,16 @@
         <v>0.0001</v>
       </c>
       <c r="I32" t="n">
-        <v>0.733</v>
+        <v>0.7688</v>
       </c>
       <c r="J32" t="n">
-        <v>0.0154</v>
+        <v>0.0114</v>
       </c>
       <c r="K32" t="n">
-        <v>0.7213000000000001</v>
+        <v>0.7271</v>
       </c>
       <c r="L32" t="n">
-        <v>1.522</v>
+        <v>1.6457</v>
       </c>
       <c r="M32" t="n">
         <v>10</v>
@@ -4945,13 +4945,13 @@
         <v>9</v>
       </c>
       <c r="O32" t="n">
-        <v>-0.0687</v>
+        <v>0.0448</v>
       </c>
       <c r="P32" t="n">
-        <v>0.261</v>
+        <v>0.3346</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.3297</v>
+        <v>0.2899</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -4969,18 +4969,18 @@
         </is>
       </c>
       <c r="U32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V32" t="n">
-        <v>66.66670000000001</v>
+        <v>55.5556</v>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2013; 2014; 2015; 2018; 2019; 2021</t>
+          <t>2014; 2015; 2018; 2019; 2021</t>
         </is>
       </c>
       <c r="X32" t="n">
-        <v>0.6485</v>
+        <v>0.7779</v>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
         <v>-0.0002</v>
       </c>
       <c r="I33" t="n">
-        <v>0.3806</v>
+        <v>0.2349</v>
       </c>
       <c r="J33" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.171</v>
       </c>
       <c r="K33" t="n">
-        <v>0.2504</v>
+        <v>0.2341</v>
       </c>
       <c r="L33" t="n">
-        <v>2.1781</v>
+        <v>2.2846</v>
       </c>
       <c r="M33" t="n">
         <v>10</v>
@@ -5046,13 +5046,13 @@
         <v>9</v>
       </c>
       <c r="O33" t="n">
-        <v>0.7872</v>
+        <v>0.8834</v>
       </c>
       <c r="P33" t="n">
-        <v>0.7539</v>
+        <v>0.8046</v>
       </c>
       <c r="Q33" t="n">
-        <v>-0.0333</v>
+        <v>-0.0788</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
@@ -5081,7 +5081,7 @@
         </is>
       </c>
       <c r="X33" t="n">
-        <v>0.2604</v>
+        <v>0.1309</v>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
@@ -5129,16 +5129,16 @@
         <v>-0.0003</v>
       </c>
       <c r="I34" t="n">
-        <v>0.2759</v>
+        <v>0.1872</v>
       </c>
       <c r="J34" t="n">
-        <v>0.3706</v>
+        <v>0.4914</v>
       </c>
       <c r="K34" t="n">
-        <v>0.1879</v>
+        <v>0.1743</v>
       </c>
       <c r="L34" t="n">
-        <v>1.5102</v>
+        <v>1.4414</v>
       </c>
       <c r="M34" t="n">
         <v>5</v>
@@ -5147,13 +5147,13 @@
         <v>4</v>
       </c>
       <c r="O34" t="n">
-        <v>0.4199</v>
+        <v>0.3979</v>
       </c>
       <c r="P34" t="n">
-        <v>0.3972</v>
+        <v>0.3535</v>
       </c>
       <c r="Q34" t="n">
-        <v>-0.0226</v>
+        <v>-0.0445</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
@@ -5182,7 +5182,7 @@
         </is>
       </c>
       <c r="X34" t="n">
-        <v>0.3381</v>
+        <v>0.2234</v>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
@@ -5227,19 +5227,19 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.0001</v>
+        <v>-0.0001</v>
       </c>
       <c r="I35" t="n">
-        <v>0.2643</v>
+        <v>0.3624</v>
       </c>
       <c r="J35" t="n">
-        <v>0.1738</v>
+        <v>0.1194</v>
       </c>
       <c r="K35" t="n">
-        <v>0.1676</v>
+        <v>0.163</v>
       </c>
       <c r="L35" t="n">
-        <v>1.8078</v>
+        <v>1.616</v>
       </c>
       <c r="M35" t="n">
         <v>9</v>
@@ -5248,13 +5248,13 @@
         <v>9</v>
       </c>
       <c r="O35" t="n">
-        <v>0.5274</v>
+        <v>0.5576</v>
       </c>
       <c r="P35" t="n">
-        <v>0.58</v>
+        <v>0.4685</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.0526</v>
+        <v>-0.0892</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
@@ -5283,7 +5283,7 @@
         </is>
       </c>
       <c r="X35" t="n">
-        <v>0.2936</v>
+        <v>0.3557</v>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
@@ -5328,19 +5328,19 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>-0.0001</v>
       </c>
       <c r="I36" t="n">
-        <v>0.9258</v>
+        <v>0.5407999999999999</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0013</v>
+        <v>0.0557</v>
       </c>
       <c r="K36" t="n">
-        <v>0.2388</v>
+        <v>0.2253</v>
       </c>
       <c r="L36" t="n">
-        <v>1.5361</v>
+        <v>1.6359</v>
       </c>
       <c r="M36" t="n">
         <v>9</v>
@@ -5349,13 +5349,13 @@
         <v>9</v>
       </c>
       <c r="O36" t="n">
-        <v>0.3482</v>
+        <v>0.4878</v>
       </c>
       <c r="P36" t="n">
-        <v>0.4013</v>
+        <v>0.4652</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.0532</v>
+        <v>-0.0227</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
@@ -5364,11 +5364,13 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T36" t="n">
-        <v>2.0014</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U36" t="n">
         <v>1</v>
@@ -5380,7 +5382,7 @@
         <v>2021</v>
       </c>
       <c r="X36" t="n">
-        <v>0.8378</v>
+        <v>0.4746</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
@@ -5428,16 +5430,16 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0572</v>
+        <v>0.6701</v>
       </c>
       <c r="J37" t="n">
-        <v>0.1616</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="K37" t="n">
-        <v>0.1699</v>
+        <v>0.2092</v>
       </c>
       <c r="L37" t="n">
-        <v>1.165</v>
+        <v>1.2156</v>
       </c>
       <c r="M37" t="n">
         <v>23</v>
@@ -5446,13 +5448,13 @@
         <v>23</v>
       </c>
       <c r="O37" t="n">
-        <v>-0.0077</v>
+        <v>0.0558</v>
       </c>
       <c r="P37" t="n">
-        <v>0.1391</v>
+        <v>0.1755</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.1469</v>
+        <v>0.1197</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
@@ -5461,11 +5463,13 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T37" t="n">
-        <v>1.9986</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U37" t="n">
         <v>6</v>
@@ -5475,15 +5479,15 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>2000; 2002; 2009; 2010; 2015; 2016</t>
+          <t>2000; 2002; 2003; 2004; 2015; 2016</t>
         </is>
       </c>
       <c r="X37" t="n">
-        <v>0.0495</v>
+        <v>0.5790999999999999</v>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
@@ -5520,23 +5524,23 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>decreasing</t>
         </is>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0.109</v>
+        <v>0.0215</v>
       </c>
       <c r="J38" t="n">
-        <v>0.1126</v>
+        <v>0.2177</v>
       </c>
       <c r="K38" t="n">
-        <v>0.1418</v>
+        <v>0.1465</v>
       </c>
       <c r="L38" t="n">
-        <v>1.2889</v>
+        <v>1.3763</v>
       </c>
       <c r="M38" t="n">
         <v>24</v>
@@ -5545,13 +5549,13 @@
         <v>23</v>
       </c>
       <c r="O38" t="n">
-        <v>0.2568</v>
+        <v>0.3718</v>
       </c>
       <c r="P38" t="n">
-        <v>0.2428</v>
+        <v>0.3073</v>
       </c>
       <c r="Q38" t="n">
-        <v>-0.014</v>
+        <v>-0.0645</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
@@ -5564,7 +5568,7 @@
         </is>
       </c>
       <c r="T38" t="n">
-        <v>3.0007</v>
+        <v>23.0007</v>
       </c>
       <c r="U38" t="n">
         <v>1</v>
@@ -5576,11 +5580,11 @@
         <v>2020</v>
       </c>
       <c r="X38" t="n">
-        <v>0.07729999999999999</v>
+        <v>0.0156</v>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>non-directional</t>
+          <t>decreasing</t>
         </is>
       </c>
     </row>
@@ -5621,19 +5625,19 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>-0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="I39" t="n">
-        <v>0.743</v>
+        <v>0.5614</v>
       </c>
       <c r="J39" t="n">
-        <v>0.0413</v>
+        <v>0.1238</v>
       </c>
       <c r="K39" t="n">
-        <v>0.1965</v>
+        <v>0.1926</v>
       </c>
       <c r="L39" t="n">
-        <v>1.5264</v>
+        <v>1.6056</v>
       </c>
       <c r="M39" t="n">
         <v>5</v>
@@ -5642,13 +5646,13 @@
         <v>4</v>
       </c>
       <c r="O39" t="n">
-        <v>0.3815</v>
+        <v>0.3652</v>
       </c>
       <c r="P39" t="n">
-        <v>0.4052</v>
+        <v>0.4581</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.0237</v>
+        <v>0.0929</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -5677,7 +5681,7 @@
         </is>
       </c>
       <c r="X39" t="n">
-        <v>0.7864</v>
+        <v>0.5778</v>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
@@ -5718,23 +5722,23 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H40" t="n">
         <v>-0.0001</v>
       </c>
       <c r="I40" t="n">
-        <v>0.4752</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="J40" t="n">
-        <v>0.06560000000000001</v>
+        <v>0.0433</v>
       </c>
       <c r="K40" t="n">
-        <v>0.3018</v>
+        <v>0.2891</v>
       </c>
       <c r="L40" t="n">
-        <v>1.734</v>
+        <v>1.8703</v>
       </c>
       <c r="M40" t="n">
         <v>10</v>
@@ -5743,13 +5747,13 @@
         <v>9</v>
       </c>
       <c r="O40" t="n">
-        <v>0.5159</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="P40" t="n">
-        <v>0.5088</v>
+        <v>0.5885</v>
       </c>
       <c r="Q40" t="n">
-        <v>-0.0071</v>
+        <v>0.0285</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
@@ -5778,7 +5782,7 @@
         </is>
       </c>
       <c r="X40" t="n">
-        <v>0.4956</v>
+        <v>0.5803</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
@@ -5823,19 +5827,19 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>-0.0005</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0415</v>
+        <v>0.0278</v>
       </c>
       <c r="J41" t="n">
-        <v>0.4239</v>
+        <v>0.4735</v>
       </c>
       <c r="K41" t="n">
-        <v>0.3842</v>
+        <v>0.406</v>
       </c>
       <c r="L41" t="n">
-        <v>2.1678</v>
+        <v>2.3611</v>
       </c>
       <c r="M41" t="n">
         <v>10</v>
@@ -5844,13 +5848,13 @@
         <v>9</v>
       </c>
       <c r="O41" t="n">
-        <v>1.0566</v>
+        <v>1.1862</v>
       </c>
       <c r="P41" t="n">
-        <v>0.7064</v>
+        <v>0.7828000000000001</v>
       </c>
       <c r="Q41" t="n">
-        <v>-0.3502</v>
+        <v>-0.4035</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
@@ -5863,7 +5867,7 @@
         </is>
       </c>
       <c r="T41" t="n">
-        <v>9.0021</v>
+        <v>4</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
@@ -5877,7 +5881,7 @@
         </is>
       </c>
       <c r="X41" t="n">
-        <v>0.0266</v>
+        <v>0.0173</v>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
@@ -5922,19 +5926,19 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>-0.0003</v>
+        <v>-0.0001</v>
       </c>
       <c r="I42" t="n">
-        <v>0.3918</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="J42" t="n">
-        <v>0.2493</v>
+        <v>0.0609</v>
       </c>
       <c r="K42" t="n">
-        <v>0.1912</v>
+        <v>0.1426</v>
       </c>
       <c r="L42" t="n">
-        <v>1.7999</v>
+        <v>1.723</v>
       </c>
       <c r="M42" t="n">
         <v>5</v>
@@ -5943,13 +5947,13 @@
         <v>4</v>
       </c>
       <c r="O42" t="n">
-        <v>0.5924</v>
+        <v>0.546</v>
       </c>
       <c r="P42" t="n">
-        <v>0.5725</v>
+        <v>0.536</v>
       </c>
       <c r="Q42" t="n">
-        <v>-0.0199</v>
+        <v>-0.01</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
@@ -5978,7 +5982,7 @@
         </is>
       </c>
       <c r="X42" t="n">
-        <v>0.438</v>
+        <v>0.6896</v>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
@@ -6019,23 +6023,23 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>-0.0001</v>
       </c>
       <c r="I43" t="n">
-        <v>0.8786</v>
+        <v>0.7403</v>
       </c>
       <c r="J43" t="n">
-        <v>0.0036</v>
+        <v>0.0167</v>
       </c>
       <c r="K43" t="n">
-        <v>0.326</v>
+        <v>0.2891</v>
       </c>
       <c r="L43" t="n">
-        <v>1.8571</v>
+        <v>2.0255</v>
       </c>
       <c r="M43" t="n">
         <v>9</v>
@@ -6044,13 +6048,13 @@
         <v>9</v>
       </c>
       <c r="O43" t="n">
-        <v>0.4284</v>
+        <v>0.6326000000000001</v>
       </c>
       <c r="P43" t="n">
-        <v>0.5736</v>
+        <v>0.6687</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.1452</v>
+        <v>0.0362</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
@@ -6079,7 +6083,7 @@
         </is>
       </c>
       <c r="X43" t="n">
-        <v>0.8431999999999999</v>
+        <v>0.6166</v>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
@@ -6120,23 +6124,23 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H44" t="n">
         <v>0.0003</v>
       </c>
       <c r="I44" t="n">
-        <v>0.3224</v>
+        <v>0.3883</v>
       </c>
       <c r="J44" t="n">
-        <v>0.1393</v>
+        <v>0.1078</v>
       </c>
       <c r="K44" t="n">
-        <v>0.3059</v>
+        <v>0.2872</v>
       </c>
       <c r="L44" t="n">
-        <v>2.6194</v>
+        <v>2.9202</v>
       </c>
       <c r="M44" t="n">
         <v>9</v>
@@ -6145,17 +6149,17 @@
         <v>9</v>
       </c>
       <c r="O44" t="n">
-        <v>0.72</v>
+        <v>0.8683</v>
       </c>
       <c r="P44" t="n">
-        <v>0.9232</v>
+        <v>1.0354</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.2032</v>
+        <v>0.167</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>accurate</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -6180,7 +6184,7 @@
         </is>
       </c>
       <c r="X44" t="n">
-        <v>0.2542</v>
+        <v>0.3338</v>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
@@ -6228,16 +6232,16 @@
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>0.2123</v>
+        <v>0.1707</v>
       </c>
       <c r="J45" t="n">
-        <v>0.073</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="K45" t="n">
-        <v>0.1289</v>
+        <v>0.2062</v>
       </c>
       <c r="L45" t="n">
-        <v>1.3897</v>
+        <v>1.4596</v>
       </c>
       <c r="M45" t="n">
         <v>23</v>
@@ -6246,13 +6250,13 @@
         <v>23</v>
       </c>
       <c r="O45" t="n">
-        <v>0.3181</v>
+        <v>0.41</v>
       </c>
       <c r="P45" t="n">
-        <v>0.3206</v>
+        <v>0.3588</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.0025</v>
+        <v>-0.0513</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -6261,13 +6265,11 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T45" t="n">
+        <v>3.0007</v>
       </c>
       <c r="U45" t="n">
         <v>2</v>
@@ -6281,7 +6283,7 @@
         </is>
       </c>
       <c r="X45" t="n">
-        <v>0.1823</v>
+        <v>0.1266</v>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
@@ -6923,31 +6925,31 @@
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>0.1117</v>
+        <v>0.3808</v>
       </c>
       <c r="J52" t="n">
-        <v>0.0796</v>
+        <v>0.0286</v>
       </c>
       <c r="K52" t="n">
-        <v>0.3471</v>
+        <v>0.3443</v>
       </c>
       <c r="L52" t="n">
-        <v>1.5341</v>
+        <v>1.4784</v>
       </c>
       <c r="M52" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="N52" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="O52" t="n">
         <v>0.3503</v>
       </c>
       <c r="P52" t="n">
-        <v>0.3727</v>
+        <v>0.3388</v>
       </c>
       <c r="Q52" t="n">
-        <v>0.0224</v>
+        <v>-0.0115</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
@@ -6965,18 +6967,18 @@
         </is>
       </c>
       <c r="U52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V52" t="n">
-        <v>21.875</v>
+        <v>21.4286</v>
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>1991; 1999; 2001; 2006; 2007; 2018; 2019</t>
+          <t>1991; 1999; 2001; 2006; 2007; 2018</t>
         </is>
       </c>
       <c r="X52" t="n">
-        <v>0.1141</v>
+        <v>0.3762</v>
       </c>
       <c r="Y52" t="inlineStr">
         <is>
@@ -7017,38 +7019,38 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>0.0457</v>
+        <v>0.2291</v>
       </c>
       <c r="J53" t="n">
-        <v>0.1227</v>
+        <v>0.0531</v>
       </c>
       <c r="K53" t="n">
-        <v>0.3335</v>
+        <v>0.333</v>
       </c>
       <c r="L53" t="n">
-        <v>1.5951</v>
+        <v>1.5294</v>
       </c>
       <c r="M53" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="N53" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="O53" t="n">
         <v>0.4244</v>
       </c>
       <c r="P53" t="n">
-        <v>0.4146</v>
+        <v>0.3734</v>
       </c>
       <c r="Q53" t="n">
-        <v>-0.0098</v>
+        <v>-0.051</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -7057,29 +7059,31 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T53" t="n">
-        <v>32</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V53" t="n">
-        <v>18.75</v>
+        <v>17.8571</v>
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>1994; 1995; 1999; 2000; 2018; 2019</t>
+          <t>1994; 1995; 1999; 2000; 2018</t>
         </is>
       </c>
       <c r="X53" t="n">
-        <v>0.0465</v>
+        <v>0.2542</v>
       </c>
       <c r="Y53" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
@@ -7123,16 +7127,16 @@
         <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>0.7957</v>
+        <v>0.7714</v>
       </c>
       <c r="J54" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.1235</v>
       </c>
       <c r="K54" t="n">
-        <v>0.1908</v>
+        <v>0.1919</v>
       </c>
       <c r="L54" t="n">
-        <v>1.2013</v>
+        <v>1.2066</v>
       </c>
       <c r="M54" t="n">
         <v>3</v>
@@ -7144,10 +7148,10 @@
         <v>0.1395</v>
       </c>
       <c r="P54" t="n">
-        <v>0.1705</v>
+        <v>0.1746</v>
       </c>
       <c r="Q54" t="n">
-        <v>0.031</v>
+        <v>0.0351</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
@@ -7174,7 +7178,7 @@
         <v>1995</v>
       </c>
       <c r="X54" t="n">
-        <v>0.7694</v>
+        <v>0.7477</v>
       </c>
       <c r="Y54" t="inlineStr">
         <is>
@@ -7222,31 +7226,31 @@
         <v>0.0001</v>
       </c>
       <c r="I55" t="n">
-        <v>0.0014</v>
+        <v>0.013</v>
       </c>
       <c r="J55" t="n">
-        <v>0.2828</v>
+        <v>0.2074</v>
       </c>
       <c r="K55" t="n">
-        <v>0.2879</v>
+        <v>0.2924</v>
       </c>
       <c r="L55" t="n">
-        <v>1.404</v>
+        <v>1.3536</v>
       </c>
       <c r="M55" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="N55" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="O55" t="n">
         <v>0.124</v>
       </c>
       <c r="P55" t="n">
-        <v>0.3033</v>
+        <v>0.2669</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.1793</v>
+        <v>0.1429</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
@@ -7262,18 +7266,18 @@
         <v>24</v>
       </c>
       <c r="U55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V55" t="n">
         <v>25</v>
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>1991; 1992; 1994; 1995; 1999; 2001; 2018; 2019</t>
+          <t>1991; 1992; 1994; 1995; 1999; 2001; 2018</t>
         </is>
       </c>
       <c r="X55" t="n">
-        <v>0.001</v>
+        <v>0.0143</v>
       </c>
       <c r="Y55" t="inlineStr">
         <is>
@@ -7314,65 +7318,67 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H56" t="n">
         <v>0.0001</v>
       </c>
       <c r="I56" t="n">
-        <v>0.0346</v>
+        <v>0.3818</v>
       </c>
       <c r="J56" t="n">
-        <v>0.145</v>
+        <v>0.0295</v>
       </c>
       <c r="K56" t="n">
-        <v>1.2549</v>
+        <v>0.7547</v>
       </c>
       <c r="L56" t="n">
-        <v>1.0481</v>
+        <v>1.3384</v>
       </c>
       <c r="M56" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="N56" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="O56" t="n">
-        <v>-0.8034</v>
+        <v>-0.1102</v>
       </c>
       <c r="P56" t="n">
-        <v>-0.5538999999999999</v>
+        <v>-0.1218</v>
       </c>
       <c r="Q56" t="n">
-        <v>0.2495</v>
+        <v>-0.0116</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>accurate</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T56" t="n">
-        <v>32</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U56" t="n">
         <v>15</v>
       </c>
       <c r="V56" t="n">
-        <v>50</v>
+        <v>55.5556</v>
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>1992; 1993; 1998; 1999; 2003; 2005; 2006; 2007; 2010; 2011; 2012; 2014; 2016; 2017; 2022</t>
+          <t>1992; 1993; 1995; 1996; 1997; 1999; 2002; 2005; 2006; 2007; 2010; 2011; 2012; 2014; 2016</t>
         </is>
       </c>
       <c r="X56" t="n">
-        <v>0.0557</v>
+        <v>0.3001</v>
       </c>
       <c r="Y56" t="inlineStr">
         <is>
@@ -10467,7 +10473,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -10478,10 +10484,10 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.026596</v>
+        <v>0.018233</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2979</v>
+        <v>0.1816</v>
       </c>
       <c r="J4" t="n">
         <v>5</v>
@@ -10778,10 +10784,10 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.0339</v>
+        <v>0.036039</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3906</v>
+        <v>0.445</v>
       </c>
       <c r="J11" t="n">
         <v>5</v>
@@ -10820,10 +10826,10 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>-0.002137</v>
+        <v>-0.001531</v>
       </c>
       <c r="I12" t="n">
-        <v>0.9655</v>
+        <v>0.9768</v>
       </c>
       <c r="J12" t="n">
         <v>5</v>
@@ -10862,10 +10868,10 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-0.066248</v>
+        <v>-0.083858</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3295</v>
+        <v>0.1855</v>
       </c>
       <c r="J13" t="n">
         <v>5</v>
@@ -10904,10 +10910,10 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.013874</v>
+        <v>0.057858</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8129</v>
+        <v>0.3101</v>
       </c>
       <c r="J14" t="n">
         <v>5</v>
@@ -10946,10 +10952,10 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>-0.019641</v>
+        <v>-0.030688</v>
       </c>
       <c r="I15" t="n">
-        <v>0.7229</v>
+        <v>0.5385</v>
       </c>
       <c r="J15" t="n">
         <v>5</v>
@@ -10988,10 +10994,10 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>-0.01039</v>
+        <v>-0.027891</v>
       </c>
       <c r="I16" t="n">
-        <v>0.8439</v>
+        <v>0.6272</v>
       </c>
       <c r="J16" t="n">
         <v>5</v>
@@ -11030,10 +11036,10 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>-0.194572</v>
+        <v>-0.265037</v>
       </c>
       <c r="I17" t="n">
-        <v>0.0155</v>
+        <v>0.0063</v>
       </c>
       <c r="J17" t="n">
         <v>5</v>
@@ -11064,21 +11070,21 @@
         <v>23</v>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1999; 2011</t>
+          <t>2001; 2004; 2015</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>-0.132096; 0.041836; -0.008065</t>
+          <t>-0.07757; 0.257033; -0.005213; -0.045065</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>NaN; 6e-04; 0.6891</t>
+          <t>0.2796; 0.039; 0.8061; 0.2125</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -11110,18 +11116,20 @@
         <v>24</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>-0.004744</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0.07770000000000001</v>
+        <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2005</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>-0.038159; -0.001718</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>0.0048; 0.7783</t>
+        </is>
       </c>
       <c r="J19" t="n">
         <v>5</v>
@@ -11160,10 +11168,10 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>-0.032188</v>
+        <v>-0.017448</v>
       </c>
       <c r="I20" t="n">
-        <v>0.4005</v>
+        <v>0.6807</v>
       </c>
       <c r="J20" t="n">
         <v>5</v>
@@ -11202,10 +11210,10 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0.0046</v>
+        <v>-0.009150999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>0.8794</v>
+        <v>0.7952</v>
       </c>
       <c r="J21" t="n">
         <v>5</v>
@@ -11244,10 +11252,10 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>-0.019774</v>
+        <v>-0.02591</v>
       </c>
       <c r="I22" t="n">
-        <v>0.7307</v>
+        <v>0.7068</v>
       </c>
       <c r="J22" t="n">
         <v>5</v>
@@ -11286,10 +11294,10 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>0.033756</v>
+        <v>0.003813</v>
       </c>
       <c r="I23" t="n">
-        <v>0.6383</v>
+        <v>0.9637</v>
       </c>
       <c r="J23" t="n">
         <v>5</v>
@@ -11328,10 +11336,10 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>-0.034008</v>
+        <v>-0.0291</v>
       </c>
       <c r="I24" t="n">
-        <v>0.3696</v>
+        <v>0.4763</v>
       </c>
       <c r="J24" t="n">
         <v>5</v>
@@ -11370,10 +11378,10 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>0.030953</v>
+        <v>0.019832</v>
       </c>
       <c r="I25" t="n">
-        <v>0.5165999999999999</v>
+        <v>0.6737</v>
       </c>
       <c r="J25" t="n">
         <v>5</v>
@@ -11412,10 +11420,10 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0.034591</v>
+        <v>0.022429</v>
       </c>
       <c r="I26" t="n">
-        <v>0.4683</v>
+        <v>0.7030999999999999</v>
       </c>
       <c r="J26" t="n">
         <v>5</v>
@@ -11446,21 +11454,19 @@
         <v>23</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2008; 2010</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2018</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>-0.011135; 0.058006; -0.038235</t>
+          <t>0.005961; -0.113073</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>0.1133; NaN; 0.1589</t>
+          <t>0.461; NaN</t>
         </is>
       </c>
       <c r="J27" t="n">
@@ -11500,10 +11506,10 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>-0.002127</v>
+        <v>-0.003678</v>
       </c>
       <c r="I28" t="n">
-        <v>0.542</v>
+        <v>0.3208</v>
       </c>
       <c r="J28" t="n">
         <v>5</v>
@@ -11542,10 +11548,10 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>-0.194584</v>
+        <v>-0.217598</v>
       </c>
       <c r="I29" t="n">
-        <v>0.0035</v>
+        <v>0.0939</v>
       </c>
       <c r="J29" t="n">
         <v>5</v>
@@ -11584,10 +11590,10 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0.044922</v>
+        <v>0.042229</v>
       </c>
       <c r="I30" t="n">
-        <v>0.7331</v>
+        <v>0.7689</v>
       </c>
       <c r="J30" t="n">
         <v>5</v>
@@ -11626,10 +11632,10 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>-0.056162</v>
+        <v>-0.07308000000000001</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3805</v>
+        <v>0.2348</v>
       </c>
       <c r="J31" t="n">
         <v>5</v>
@@ -11668,10 +11674,10 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>-0.109183</v>
+        <v>-0.111333</v>
       </c>
       <c r="I32" t="n">
-        <v>0.2762</v>
+        <v>0.1875</v>
       </c>
       <c r="J32" t="n">
         <v>5</v>
@@ -11710,10 +11716,10 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>0.043025</v>
+        <v>-0.031022</v>
       </c>
       <c r="I33" t="n">
-        <v>0.2644</v>
+        <v>0.3624</v>
       </c>
       <c r="J33" t="n">
         <v>5</v>
@@ -11752,10 +11758,10 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>-0.004561</v>
+        <v>-0.029662</v>
       </c>
       <c r="I34" t="n">
-        <v>0.9257</v>
+        <v>0.5407</v>
       </c>
       <c r="J34" t="n">
         <v>5</v>
@@ -11794,10 +11800,10 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0.011601</v>
+        <v>0.003481</v>
       </c>
       <c r="I35" t="n">
-        <v>0.0572</v>
+        <v>0.67</v>
       </c>
       <c r="J35" t="n">
         <v>5</v>
@@ -11831,16 +11837,16 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>-0.005586; NA</t>
+          <t>-0.001469; -0.12574</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>0.3057; NA</t>
+          <t>0.8258; 0.0232</t>
         </is>
       </c>
       <c r="J36" t="n">
@@ -11880,10 +11886,10 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>-0.038478</v>
+        <v>0.068858</v>
       </c>
       <c r="I37" t="n">
-        <v>0.7436</v>
+        <v>0.5612</v>
       </c>
       <c r="J37" t="n">
         <v>5</v>
@@ -11922,10 +11928,10 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>-0.044229</v>
+        <v>-0.037132</v>
       </c>
       <c r="I38" t="n">
-        <v>0.4754</v>
+        <v>0.5643</v>
       </c>
       <c r="J38" t="n">
         <v>5</v>
@@ -11956,20 +11962,18 @@
         <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2015</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>-0.502204; -0.297546</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>0.1815; 0.1516</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>-0.217907</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.0278</v>
       </c>
       <c r="J39" t="n">
         <v>5</v>
@@ -12008,10 +12012,10 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>-0.108577</v>
+        <v>-0.038331</v>
       </c>
       <c r="I40" t="n">
-        <v>0.3922</v>
+        <v>0.6892</v>
       </c>
       <c r="J40" t="n">
         <v>5</v>
@@ -12050,10 +12054,10 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.012361</v>
+        <v>-0.025773</v>
       </c>
       <c r="I41" t="n">
-        <v>0.8783</v>
+        <v>0.7405</v>
       </c>
       <c r="J41" t="n">
         <v>5</v>
@@ -12092,10 +12096,10 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>0.101924</v>
+        <v>0.093847</v>
       </c>
       <c r="I42" t="n">
-        <v>0.3224</v>
+        <v>0.3883</v>
       </c>
       <c r="J42" t="n">
         <v>5</v>
@@ -12126,18 +12130,20 @@
         <v>23</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H43" t="n">
-        <v>-0.007059</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0.2124</v>
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2015</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>0.003826; -0.070093</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>0.7799; 0.285</t>
+        </is>
       </c>
       <c r="J43" t="n">
         <v>5</v>
@@ -12425,25 +12431,21 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F50" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2010; 2011</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>-0.010684; NA; 0.042017</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>0.5202; NA; 0.5095</t>
-        </is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>0.010103</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.3808</v>
       </c>
       <c r="J50" t="n">
         <v>5</v>
@@ -12471,25 +12473,21 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2007; 2010</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>-0.008441; 0.160135; 0.046089</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>0.7031; 0.6703; 0.3779</t>
-        </is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>0.013785</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.2291</v>
       </c>
       <c r="J51" t="n">
         <v>5</v>
@@ -12517,7 +12515,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F52" t="n">
         <v>2</v>
@@ -12529,12 +12527,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>0.009502; 0.060339; 0.003446</t>
+          <t>0.008891; 0.061889; -0.023046</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>0.5452; 0.2825; 0.9511</t>
+          <t>0.5705; 0.291; 0.8868</t>
         </is>
       </c>
       <c r="J52" t="n">
@@ -12563,7 +12561,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -12574,10 +12572,10 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>0.053197</v>
+        <v>0.02111</v>
       </c>
       <c r="I53" t="n">
-        <v>0.0346</v>
+        <v>0.3817</v>
       </c>
       <c r="J53" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
Table 1 / S1: one row per dataset when a dataset spans several EDI entities
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1466,17 +1466,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BNZ</t>
+          <t>MCM</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bonanza Creek</t>
+          <t>McMurdo Dry Valleys</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Boreal forest / permafrost tundra</t>
+          <t>Polar desert soil</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1486,17 +1486,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CiPEHR (Carbon in Permafrost Experimental Heating Research)</t>
+          <t>Stoichiometry experiment (Bonney and Fryxell basins)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Warming (soil and air)</t>
+          <t>Nutrient addition (C, N, P)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Net ecosystem exchange</t>
+          <t>Soil CO2 flux</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1506,42 +1506,40 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2009-2021</t>
+          <t>2003-2010</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>13</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>3 (6)</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>knb-lter-bnz.481.23</t>
+          <t>knb-lter-mcm.4014.5</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Rodenhizer, H. G., Mauritz, M., Taylor, M., Ledman, J., Natali, S. &amp; Schuur, E. (2022). Data from: “Eight Mile Lake Research Watershed, Carbon in Permafrost Experimental Heating Research (CiPEHR): Half-hourly growing season, chamber-based, CO2 flux data, 2009-2021 ver 23.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5ee6a71835606934afda8e3eb9a38763</t>
+          <t>Virginia, R. &amp; Wall, D. (2016). Data from: “McMurdo Dry Valleys Stoichiometry Experiment - CO2 ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f2c3854f11c24c54be3f3828c130746f</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BNZ</t>
+          <t>NWT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bonanza Creek</t>
+          <t>Niwot Ridge</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Boreal forest / permafrost tundra</t>
+          <t>Alpine tundra</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1551,362 +1549,104 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CiPEHR (Carbon in Permafrost Experimental Heating Research)</t>
+          <t>Snow x N x temperature experiment (Niwot Saddle)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Warming (soil and air)</t>
+          <t>Fertilization (N; ambient snow and temperature plots)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Net ecosystem exchange</t>
+          <t>Aboveground biomass (g m-2)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Flux</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2009-2021</t>
+          <t>2006-2019</t>
         </is>
       </c>
       <c r="J20" t="n">
         <v>13</v>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>3 (6)</t>
-        </is>
+      <c r="K20" t="n">
+        <v>1</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>knb-lter-bnz.481.23</t>
+          <t>knb-lter-nwt.13.7</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Rodenhizer, H. G., Mauritz, M., Taylor, M., Ledman, J., Natali, S. &amp; Schuur, E. (2022). Data from: “Eight Mile Lake Research Watershed, Carbon in Permafrost Experimental Heating Research (CiPEHR): Half-hourly growing season, chamber-based, CO2 flux data, 2009-2021 ver 23.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5ee6a71835606934afda8e3eb9a38763</t>
+          <t>Suding, K. N., Smith, J. G. &amp; Ashton, I. W. (2024). Data from: “Increased temperature, N and snowpack experiment for north of saddle, 2006 - ongoing. ver 7.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/caacfd0b6e32b5a72f8fe3904ca897bf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BNZ</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bonanza Creek</t>
+          <t>Central Arizona-Phoenix</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Boreal forest / permafrost tundra</t>
+          <t>Sonoran Desert</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Tundra</t>
+          <t>Urban</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CiPEHR (Carbon in Permafrost Experimental Heating Research)</t>
+          <t>Desert Fertilization Experiment (CNdep)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Warming (soil and air)</t>
+          <t>Fertilization (N, P)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Net ecosystem exchange</t>
+          <t>Aboveground biomass (g m-2)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Flux</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2009-2021</t>
+          <t>2008-2024</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>13</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>3 (6)</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>knb-lter-bnz.481.23</t>
+          <t>knb-lter-cap.632.17</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
-        <is>
-          <t>Rodenhizer, H. G., Mauritz, M., Taylor, M., Ledman, J., Natali, S. &amp; Schuur, E. (2022). Data from: “Eight Mile Lake Research Watershed, Carbon in Permafrost Experimental Heating Research (CiPEHR): Half-hourly growing season, chamber-based, CO2 flux data, 2009-2021 ver 23.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5ee6a71835606934afda8e3eb9a38763</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>BNZ</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Bonanza Creek</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Boreal forest / permafrost tundra</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Tundra</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>CiPEHR (Carbon in Permafrost Experimental Heating Research)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Warming (soil and air)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Net ecosystem exchange</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Flux</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>2009-2021</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>13</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>3 (6)</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>knb-lter-bnz.481.23</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Rodenhizer, H. G., Mauritz, M., Taylor, M., Ledman, J., Natali, S. &amp; Schuur, E. (2022). Data from: “Eight Mile Lake Research Watershed, Carbon in Permafrost Experimental Heating Research (CiPEHR): Half-hourly growing season, chamber-based, CO2 flux data, 2009-2021 ver 23.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5ee6a71835606934afda8e3eb9a38763</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>MCM</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>McMurdo Dry Valleys</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Polar desert soil</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Tundra</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Stoichiometry experiment (Bonney and Fryxell basins)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Nutrient addition (C, N, P)</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Soil CO2 flux</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Flux</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2003-2010</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>5</v>
-      </c>
-      <c r="K23" t="n">
-        <v>5</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>knb-lter-mcm.4014.5</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Virginia, R. &amp; Wall, D. (2016). Data from: “McMurdo Dry Valleys Stoichiometry Experiment - CO2 ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f2c3854f11c24c54be3f3828c130746f</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>NWT</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Niwot Ridge</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Alpine tundra</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Tundra</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Snow x N x temperature experiment (Niwot Saddle)</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Fertilization (N; ambient snow and temperature plots)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Aboveground biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2006-2019</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>13</v>
-      </c>
-      <c r="K24" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>knb-lter-nwt.13.7</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Suding, K. N., Smith, J. G. &amp; Ashton, I. W. (2024). Data from: “Increased temperature, N and snowpack experiment for north of saddle, 2006 - ongoing. ver 7.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/caacfd0b6e32b5a72f8fe3904ca897bf</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>CAP</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Central Arizona-Phoenix</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Sonoran Desert</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Urban</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Desert Fertilization Experiment (CNdep)</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Fertilization (N, P)</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Aboveground biomass (g m-2)</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2008-2024</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>12</v>
-      </c>
-      <c r="K25" t="n">
-        <v>3</v>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>knb-lter-cap.632.17</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
         <is>
           <t>Grimm, N., Hall, S. J., Kaye, J. &amp; Allen, J. (2024). Data from: “Desert Fertilization Experiment: investigation of Sonoran desert ecosystem response to atmospheric deposition and experimental nutrient addition, ongoing since 2006 ver 17.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/fd7e336a9493e780777d97bb08ff2352</t>
         </is>

</xml_diff>

<commit_message>
Table S1 years from the paired record; captions and supplement at final numbers
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -620,11 +620,11 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2004-2020</t>
+          <t>2004-2019</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K5" t="n">
         <v>1</v>
@@ -1061,11 +1061,11 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2011-2019</t>
+          <t>2013-2019</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
         <v>1</v>
@@ -1376,11 +1376,11 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1982-2015</t>
+          <t>1983-2015</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table S2. Per-treatment statistics for the 83 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; tolerance 0.2), years to first detection of a significant trend (directional treatments only), the number, percentage (of consecutive measurement transitions), and years of sign flips, and the P-value and directional call when the trend analysis is repeated on the log response ratio.</t>
+          <t>Table S2. Per-treatment statistics for the 78 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; tolerance 0.2), years to first detection of a significant trend (directional treatments only), the number, percentage (of consecutive measurement transitions), and years of sign flips, and the P-value and directional call when the trend analysis is repeated on the log response ratio.</t>
         </is>
       </c>
     </row>
@@ -9634,7 +9634,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table S3. SiZer results for the 79 treatment-experiment combinations with at least five timepoints: number of significant slope changes at a 5-year bandwidth, the years at which they occurred, and segment slopes with P-values.</t>
+          <t>Table S3. SiZer results for the 74 treatment-experiment combinations with at least five timepoints: number of significant slope changes at a 5-year bandwidth, the years at which they occurred, and segment slopes with P-values.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Detection persistence statistics; regenerate outputs
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -557,11 +557,11 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2010-2020</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="K4" t="n">
         <v>1</v>
@@ -1194,7 +1194,7 @@
         <v>26</v>
       </c>
       <c r="K14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1661,7 +1661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y81"/>
+  <dimension ref="A1:Y80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5555,38 +5555,38 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>increasing</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.0001</v>
+        <v>0.0003</v>
       </c>
       <c r="I41" t="n">
-        <v>0.1376</v>
+        <v>0.0187</v>
       </c>
       <c r="J41" t="n">
-        <v>0.2278</v>
+        <v>0.8782</v>
       </c>
       <c r="K41" t="n">
-        <v>0.152</v>
+        <v>0.2382</v>
       </c>
       <c r="L41" t="n">
-        <v>0.855</v>
+        <v>0.8167</v>
       </c>
       <c r="M41" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N41" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="O41" t="n">
         <v>-0.3604</v>
       </c>
       <c r="P41" t="n">
-        <v>-0.17</v>
+        <v>-0.2293</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.1905</v>
+        <v>0.1311</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
@@ -5613,11 +5613,11 @@
         </is>
       </c>
       <c r="X41" t="n">
-        <v>0.1158</v>
+        <v>0.0316</v>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>non-directional</t>
+          <t>increasing</t>
         </is>
       </c>
     </row>
@@ -5661,16 +5661,16 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0.4202</v>
+        <v>0.3672</v>
       </c>
       <c r="J42" t="n">
-        <v>0.1676</v>
+        <v>0.2051</v>
       </c>
       <c r="K42" t="n">
-        <v>0.0311</v>
+        <v>0.068</v>
       </c>
       <c r="L42" t="n">
-        <v>0.9808</v>
+        <v>0.9359</v>
       </c>
       <c r="M42" t="n">
         <v>6</v>
@@ -5679,13 +5679,13 @@
         <v>6</v>
       </c>
       <c r="O42" t="n">
-        <v>-0.0334</v>
+        <v>-0.08649999999999999</v>
       </c>
       <c r="P42" t="n">
-        <v>-0.0197</v>
+        <v>-0.0703</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.0137</v>
+        <v>0.0162</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="X42" t="n">
-        <v>0.42</v>
+        <v>0.3732</v>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
@@ -5765,13 +5765,13 @@
         <v>0.0001</v>
       </c>
       <c r="J43" t="n">
-        <v>0.8475</v>
+        <v>0.8511</v>
       </c>
       <c r="K43" t="n">
-        <v>0.0484</v>
+        <v>0.0486</v>
       </c>
       <c r="L43" t="n">
-        <v>1.0136</v>
+        <v>1.0187</v>
       </c>
       <c r="M43" t="n">
         <v>11</v>
@@ -5780,13 +5780,13 @@
         <v>10</v>
       </c>
       <c r="O43" t="n">
-        <v>-0.0314</v>
+        <v>-0.0292</v>
       </c>
       <c r="P43" t="n">
-        <v>0.0125</v>
+        <v>0.0103</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.0439</v>
+        <v>0.0395</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="T43" t="n">
-        <v>6.0014</v>
+        <v>7.0007</v>
       </c>
       <c r="U43" t="n">
         <v>1</v>
@@ -5859,16 +5859,16 @@
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0142</v>
+        <v>0.017</v>
       </c>
       <c r="J44" t="n">
-        <v>0.5053</v>
+        <v>0.4866</v>
       </c>
       <c r="K44" t="n">
-        <v>0.0429</v>
+        <v>0.044</v>
       </c>
       <c r="L44" t="n">
-        <v>0.9907</v>
+        <v>0.9963</v>
       </c>
       <c r="M44" t="n">
         <v>11</v>
@@ -5877,13 +5877,13 @@
         <v>10</v>
       </c>
       <c r="O44" t="n">
-        <v>-0.0325</v>
+        <v>-0.0356</v>
       </c>
       <c r="P44" t="n">
-        <v>-0.0102</v>
+        <v>-0.0174</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.0223</v>
+        <v>0.0182</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
@@ -5910,7 +5910,7 @@
         </is>
       </c>
       <c r="X44" t="n">
-        <v>0.0154</v>
+        <v>0.0183</v>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>0.1167</v>
+        <v>0.2116</v>
       </c>
       <c r="J45" t="n">
-        <v>0.2507</v>
+        <v>0.1673</v>
       </c>
       <c r="K45" t="n">
-        <v>0.0257</v>
+        <v>0.0237</v>
       </c>
       <c r="L45" t="n">
-        <v>0.9566</v>
+        <v>0.9631</v>
       </c>
       <c r="M45" t="n">
         <v>11</v>
@@ -5976,13 +5976,13 @@
         <v>10</v>
       </c>
       <c r="O45" t="n">
-        <v>-0.0612</v>
+        <v>-0.0595</v>
       </c>
       <c r="P45" t="n">
-        <v>-0.0447</v>
+        <v>-0.0466</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.0165</v>
+        <v>0.0129</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -6000,18 +6000,18 @@
         </is>
       </c>
       <c r="U45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V45" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>2015; 2016</t>
         </is>
       </c>
       <c r="X45" t="n">
-        <v>0.1152</v>
+        <v>0.2093</v>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
@@ -6151,23 +6151,23 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H47" t="n">
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>0.2937</v>
+        <v>0.468</v>
       </c>
       <c r="J47" t="n">
-        <v>0.0458</v>
+        <v>0.0222</v>
       </c>
       <c r="K47" t="n">
-        <v>0.3465</v>
+        <v>0.2903</v>
       </c>
       <c r="L47" t="n">
-        <v>1.476</v>
+        <v>1.1699</v>
       </c>
       <c r="M47" t="n">
         <v>26</v>
@@ -6176,13 +6176,13 @@
         <v>25</v>
       </c>
       <c r="O47" t="n">
-        <v>0.4071</v>
+        <v>0.2382</v>
       </c>
       <c r="P47" t="n">
-        <v>0.3374</v>
+        <v>0.1187</v>
       </c>
       <c r="Q47" t="n">
-        <v>-0.0696</v>
+        <v>-0.1195</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
@@ -6200,18 +6200,18 @@
         </is>
       </c>
       <c r="U47" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="V47" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>1999; 2001; 2006; 2007; 2018</t>
+          <t>1994; 1995; 1996; 1998; 1999; 2001; 2005; 2007; 2009; 2010; 2012; 2013; 2015; 2016; 2018</t>
         </is>
       </c>
       <c r="X47" t="n">
-        <v>0.2917</v>
+        <v>0.4854</v>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
@@ -6256,19 +6256,19 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>0.1221</v>
+        <v>0.2603</v>
       </c>
       <c r="J48" t="n">
-        <v>0.09669999999999999</v>
+        <v>0.0525</v>
       </c>
       <c r="K48" t="n">
-        <v>0.3372</v>
+        <v>0.3045</v>
       </c>
       <c r="L48" t="n">
-        <v>1.5218</v>
+        <v>1.2125</v>
       </c>
       <c r="M48" t="n">
         <v>26</v>
@@ -6277,13 +6277,13 @@
         <v>25</v>
       </c>
       <c r="O48" t="n">
-        <v>0.3358</v>
+        <v>0.2054</v>
       </c>
       <c r="P48" t="n">
-        <v>0.3675</v>
+        <v>0.1506</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.0318</v>
+        <v>-0.0548</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -6292,25 +6292,27 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T48" t="n">
-        <v>24</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U48" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="V48" t="n">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>1994; 1995; 1999; 2000; 2018</t>
+          <t>1994; 1995; 1997; 1998; 1999; 2001; 2002; 2004; 2005; 2007; 2009; 2010; 2018</t>
         </is>
       </c>
       <c r="X48" t="n">
-        <v>0.1356</v>
+        <v>0.2865</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
@@ -6355,19 +6357,19 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I49" t="n">
-        <v>0.7714</v>
+        <v>0.6088</v>
       </c>
       <c r="J49" t="n">
-        <v>0.1235</v>
+        <v>0.3324</v>
       </c>
       <c r="K49" t="n">
-        <v>0.1919</v>
+        <v>0.2479</v>
       </c>
       <c r="L49" t="n">
-        <v>1.2066</v>
+        <v>1.1149</v>
       </c>
       <c r="M49" t="n">
         <v>3</v>
@@ -6376,13 +6378,13 @@
         <v>10</v>
       </c>
       <c r="O49" t="n">
-        <v>0.1395</v>
+        <v>0.007</v>
       </c>
       <c r="P49" t="n">
-        <v>0.1746</v>
+        <v>0.0856</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.0351</v>
+        <v>0.0785</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -6409,7 +6411,7 @@
         <v>1995</v>
       </c>
       <c r="X49" t="n">
-        <v>0.7477</v>
+        <v>0.6088</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
@@ -6454,19 +6456,19 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>0.0225</v>
+        <v>0.0202</v>
       </c>
       <c r="J50" t="n">
-        <v>0.1987</v>
+        <v>0.205</v>
       </c>
       <c r="K50" t="n">
-        <v>0.2918</v>
+        <v>0.2056</v>
       </c>
       <c r="L50" t="n">
-        <v>1.3755</v>
+        <v>1.2092</v>
       </c>
       <c r="M50" t="n">
         <v>26</v>
@@ -6475,13 +6477,13 @@
         <v>25</v>
       </c>
       <c r="O50" t="n">
-        <v>0.1768</v>
+        <v>0.1299</v>
       </c>
       <c r="P50" t="n">
-        <v>0.2834</v>
+        <v>0.1709</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.1066</v>
+        <v>0.041</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -6494,21 +6496,21 @@
         </is>
       </c>
       <c r="T50" t="n">
-        <v>21.9986</v>
+        <v>22.9979</v>
       </c>
       <c r="U50" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="V50" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>1994; 1995; 1999; 2001; 2018</t>
+          <t>1994; 1995; 1997; 1998; 1999; 2001; 2006; 2007; 2018</t>
         </is>
       </c>
       <c r="X50" t="n">
-        <v>0.0271</v>
+        <v>0.0283</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
@@ -6519,12 +6521,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>KBS</t>
+          <t>KNZ</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Kellogg Biological Station</t>
+          <t>Konza Prairie</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -6544,7 +6546,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>b m c</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -6556,35 +6558,35 @@
         <v>0.0001</v>
       </c>
       <c r="I51" t="n">
-        <v>0.4388</v>
+        <v>0.1116</v>
       </c>
       <c r="J51" t="n">
-        <v>0.0263</v>
+        <v>0.1505</v>
       </c>
       <c r="K51" t="n">
-        <v>0.7543</v>
+        <v>0.3294</v>
       </c>
       <c r="L51" t="n">
-        <v>1.3592</v>
+        <v>1.3716</v>
       </c>
       <c r="M51" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="N51" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="O51" t="n">
-        <v>-0.1345</v>
+        <v>-0.301</v>
       </c>
       <c r="P51" t="n">
-        <v>-0.1232</v>
+        <v>0.2437</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.0113</v>
+        <v>0.5447</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>wrong_direction</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -6598,22 +6600,22 @@
         </is>
       </c>
       <c r="U51" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="V51" t="n">
-        <v>54.1667</v>
+        <v>17.6471</v>
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>1995; 1996; 1997; 1999; 2002; 2005; 2006; 2007; 2010; 2011; 2012; 2014; 2016</t>
+          <t>1987; 1988; 1989</t>
         </is>
       </c>
       <c r="X51" t="n">
-        <v>0.247</v>
+        <v>0.048</v>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>non-directional</t>
+          <t>increasing</t>
         </is>
       </c>
     </row>
@@ -6645,28 +6647,28 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>b m c</t>
+          <t>b m n</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>increasing</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="I52" t="n">
-        <v>0.1116</v>
+        <v>0.0262</v>
       </c>
       <c r="J52" t="n">
-        <v>0.1505</v>
+        <v>0.2728</v>
       </c>
       <c r="K52" t="n">
-        <v>0.3294</v>
+        <v>0.3114</v>
       </c>
       <c r="L52" t="n">
-        <v>1.3716</v>
+        <v>2.611</v>
       </c>
       <c r="M52" t="n">
         <v>18</v>
@@ -6675,42 +6677,38 @@
         <v>17</v>
       </c>
       <c r="O52" t="n">
-        <v>-0.301</v>
+        <v>0.2952</v>
       </c>
       <c r="P52" t="n">
-        <v>0.2437</v>
+        <v>0.8905</v>
       </c>
       <c r="Q52" t="n">
-        <v>0.5447</v>
+        <v>0.5952</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>wrong_direction</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T52" t="n">
+        <v>16</v>
       </c>
       <c r="U52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V52" t="n">
-        <v>17.6471</v>
-      </c>
-      <c r="W52" t="inlineStr">
-        <is>
-          <t>1987; 1988; 1989</t>
-        </is>
+        <v>5.8824</v>
+      </c>
+      <c r="W52" t="n">
+        <v>1987</v>
       </c>
       <c r="X52" t="n">
-        <v>0.048</v>
+        <v>0.0193</v>
       </c>
       <c r="Y52" t="inlineStr">
         <is>
@@ -6746,28 +6744,28 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>b m n</t>
+          <t>b m n+p</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H53" t="n">
         <v>0.0002</v>
       </c>
       <c r="I53" t="n">
-        <v>0.0262</v>
+        <v>0.0819</v>
       </c>
       <c r="J53" t="n">
-        <v>0.2728</v>
+        <v>0.1773</v>
       </c>
       <c r="K53" t="n">
-        <v>0.3114</v>
+        <v>0.2955</v>
       </c>
       <c r="L53" t="n">
-        <v>2.611</v>
+        <v>2.77</v>
       </c>
       <c r="M53" t="n">
         <v>18</v>
@@ -6776,13 +6774,13 @@
         <v>17</v>
       </c>
       <c r="O53" t="n">
-        <v>0.2952</v>
+        <v>0.1663</v>
       </c>
       <c r="P53" t="n">
-        <v>0.8905</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.5952</v>
+        <v>0.7746</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -6795,19 +6793,21 @@
         </is>
       </c>
       <c r="T53" t="n">
-        <v>16</v>
+        <v>13.9986</v>
       </c>
       <c r="U53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V53" t="n">
-        <v>5.8824</v>
-      </c>
-      <c r="W53" t="n">
-        <v>1987</v>
+        <v>17.6471</v>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>1987; 1988; 1989</t>
+        </is>
       </c>
       <c r="X53" t="n">
-        <v>0.0193</v>
+        <v>0.0486</v>
       </c>
       <c r="Y53" t="inlineStr">
         <is>
@@ -6843,28 +6843,28 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>b m n+p</t>
+          <t>b m p</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="I54" t="n">
-        <v>0.0819</v>
+        <v>0.0646</v>
       </c>
       <c r="J54" t="n">
-        <v>0.1773</v>
+        <v>0.1975</v>
       </c>
       <c r="K54" t="n">
-        <v>0.2955</v>
+        <v>0.3134</v>
       </c>
       <c r="L54" t="n">
-        <v>2.77</v>
+        <v>1.3254</v>
       </c>
       <c r="M54" t="n">
         <v>18</v>
@@ -6873,17 +6873,17 @@
         <v>17</v>
       </c>
       <c r="O54" t="n">
-        <v>0.1663</v>
+        <v>-0.2252</v>
       </c>
       <c r="P54" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.2211</v>
       </c>
       <c r="Q54" t="n">
-        <v>0.7746</v>
+        <v>0.4463</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>wrong_direction</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -6892,7 +6892,7 @@
         </is>
       </c>
       <c r="T54" t="n">
-        <v>13.9986</v>
+        <v>16</v>
       </c>
       <c r="U54" t="n">
         <v>3</v>
@@ -6906,7 +6906,7 @@
         </is>
       </c>
       <c r="X54" t="n">
-        <v>0.0486</v>
+        <v>0.0329</v>
       </c>
       <c r="Y54" t="inlineStr">
         <is>
@@ -6942,47 +6942,47 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>b m p</t>
+          <t>b u c</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>increasing</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>0.0001</v>
+        <v>0.0008</v>
       </c>
       <c r="I55" t="n">
-        <v>0.0646</v>
+        <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>0.1975</v>
+        <v>0.4171</v>
       </c>
       <c r="K55" t="n">
-        <v>0.3134</v>
+        <v>1.3341</v>
       </c>
       <c r="L55" t="n">
-        <v>1.3254</v>
+        <v>3.5237</v>
       </c>
       <c r="M55" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="N55" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="O55" t="n">
-        <v>-0.2252</v>
+        <v>0.1503</v>
       </c>
       <c r="P55" t="n">
-        <v>0.2211</v>
+        <v>0.8191000000000001</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.4463</v>
+        <v>0.6688</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>wrong_direction</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -6991,21 +6991,21 @@
         </is>
       </c>
       <c r="T55" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="U55" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="V55" t="n">
-        <v>17.6471</v>
+        <v>20</v>
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>1987; 1988; 1989</t>
+          <t>1987; 1988; 1989; 2001; 2002; 2003; 2004</t>
         </is>
       </c>
       <c r="X55" t="n">
-        <v>0.0329</v>
+        <v>0</v>
       </c>
       <c r="Y55" t="inlineStr">
         <is>
@@ -7041,7 +7041,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>b u c</t>
+          <t>b u n</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -7056,28 +7056,28 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>0.4171</v>
+        <v>0.4935</v>
       </c>
       <c r="K56" t="n">
-        <v>1.3341</v>
+        <v>0.8285</v>
       </c>
       <c r="L56" t="n">
-        <v>3.5237</v>
+        <v>4.8243</v>
       </c>
       <c r="M56" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="N56" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O56" t="n">
-        <v>0.1503</v>
+        <v>0.5483</v>
       </c>
       <c r="P56" t="n">
-        <v>0.8191000000000001</v>
+        <v>1.3545</v>
       </c>
       <c r="Q56" t="n">
-        <v>0.6688</v>
+        <v>0.8062</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
@@ -7090,17 +7090,17 @@
         </is>
       </c>
       <c r="T56" t="n">
-        <v>24</v>
+        <v>5.9986</v>
       </c>
       <c r="U56" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="V56" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>1987; 1988; 1989; 2001; 2002; 2003; 2004</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="X56" t="n">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>b u n</t>
+          <t>b u n+p</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -7155,13 +7155,13 @@
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>0.4935</v>
+        <v>0.5256</v>
       </c>
       <c r="K57" t="n">
-        <v>0.8285</v>
+        <v>0.7378</v>
       </c>
       <c r="L57" t="n">
-        <v>4.8243</v>
+        <v>4.843</v>
       </c>
       <c r="M57" t="n">
         <v>31</v>
@@ -7170,13 +7170,13 @@
         <v>30</v>
       </c>
       <c r="O57" t="n">
-        <v>0.5483</v>
+        <v>0.498</v>
       </c>
       <c r="P57" t="n">
-        <v>1.3545</v>
+        <v>1.3668</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.8062</v>
+        <v>0.8688</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
@@ -7192,15 +7192,13 @@
         <v>5.9986</v>
       </c>
       <c r="U57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V57" t="n">
-        <v>0</v>
-      </c>
-      <c r="W57" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>3.3333</v>
+      </c>
+      <c r="W57" t="n">
+        <v>1987</v>
       </c>
       <c r="X57" t="n">
         <v>0</v>
@@ -7239,7 +7237,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>b u n+p</t>
+          <t>b u p</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -7248,19 +7246,19 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>0.0008</v>
+        <v>0.0003</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>0.5256</v>
+        <v>0.5885</v>
       </c>
       <c r="K58" t="n">
-        <v>0.7378</v>
+        <v>0.6942</v>
       </c>
       <c r="L58" t="n">
-        <v>4.843</v>
+        <v>2.0993</v>
       </c>
       <c r="M58" t="n">
         <v>31</v>
@@ -7269,13 +7267,13 @@
         <v>30</v>
       </c>
       <c r="O58" t="n">
-        <v>0.498</v>
+        <v>-0.0433</v>
       </c>
       <c r="P58" t="n">
-        <v>1.3668</v>
+        <v>0.5655</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.8688</v>
+        <v>0.6089</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
@@ -7288,16 +7286,18 @@
         </is>
       </c>
       <c r="T58" t="n">
-        <v>5.9986</v>
+        <v>20.9993</v>
       </c>
       <c r="U58" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V58" t="n">
-        <v>3.3333</v>
-      </c>
-      <c r="W58" t="n">
-        <v>1987</v>
+        <v>16.6667</v>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>1987; 1988; 1990; 1997; 1998</t>
+        </is>
       </c>
       <c r="X58" t="n">
         <v>0</v>
@@ -7336,74 +7336,76 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>b u p</t>
+          <t>u m c</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
+        <v>0.4047</v>
       </c>
       <c r="J59" t="n">
-        <v>0.5885</v>
+        <v>0.0438</v>
       </c>
       <c r="K59" t="n">
-        <v>0.6942</v>
+        <v>0.3028</v>
       </c>
       <c r="L59" t="n">
-        <v>2.0993</v>
+        <v>1.3126</v>
       </c>
       <c r="M59" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="N59" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="O59" t="n">
-        <v>-0.0433</v>
+        <v>-0.251</v>
       </c>
       <c r="P59" t="n">
-        <v>0.5655</v>
+        <v>0.2118</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.6089</v>
+        <v>0.4628</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>wrong_direction</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T59" t="n">
-        <v>20.9993</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U59" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V59" t="n">
-        <v>16.6667</v>
+        <v>17.6471</v>
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>1987; 1988; 1990; 1997; 1998</t>
+          <t>1987; 1988; 1989</t>
         </is>
       </c>
       <c r="X59" t="n">
-        <v>0</v>
+        <v>0.1651</v>
       </c>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
@@ -7435,7 +7437,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>u m c</t>
+          <t>u m n</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -7447,16 +7449,16 @@
         <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>0.4047</v>
+        <v>0.9584</v>
       </c>
       <c r="J60" t="n">
-        <v>0.0438</v>
+        <v>0.0002</v>
       </c>
       <c r="K60" t="n">
-        <v>0.3028</v>
+        <v>0.3639</v>
       </c>
       <c r="L60" t="n">
-        <v>1.3126</v>
+        <v>2.2465</v>
       </c>
       <c r="M60" t="n">
         <v>18</v>
@@ -7465,17 +7467,17 @@
         <v>17</v>
       </c>
       <c r="O60" t="n">
-        <v>-0.251</v>
+        <v>0.1586</v>
       </c>
       <c r="P60" t="n">
-        <v>0.2118</v>
+        <v>0.724</v>
       </c>
       <c r="Q60" t="n">
-        <v>0.4628</v>
+        <v>0.5654</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>wrong_direction</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -7489,18 +7491,16 @@
         </is>
       </c>
       <c r="U60" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V60" t="n">
-        <v>17.6471</v>
-      </c>
-      <c r="W60" t="inlineStr">
-        <is>
-          <t>1987; 1988; 1989</t>
-        </is>
+        <v>5.8824</v>
+      </c>
+      <c r="W60" t="n">
+        <v>1987</v>
       </c>
       <c r="X60" t="n">
-        <v>0.1651</v>
+        <v>0.3857</v>
       </c>
       <c r="Y60" t="inlineStr">
         <is>
@@ -7536,7 +7536,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>u m n</t>
+          <t>u m n+p</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -7545,19 +7545,19 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I61" t="n">
-        <v>0.9584</v>
+        <v>0.3927</v>
       </c>
       <c r="J61" t="n">
-        <v>0.0002</v>
+        <v>0.046</v>
       </c>
       <c r="K61" t="n">
-        <v>0.3639</v>
+        <v>0.3334</v>
       </c>
       <c r="L61" t="n">
-        <v>2.2465</v>
+        <v>2.2469</v>
       </c>
       <c r="M61" t="n">
         <v>18</v>
@@ -7566,13 +7566,13 @@
         <v>17</v>
       </c>
       <c r="O61" t="n">
-        <v>0.1586</v>
+        <v>0.1106</v>
       </c>
       <c r="P61" t="n">
-        <v>0.724</v>
+        <v>0.7204</v>
       </c>
       <c r="Q61" t="n">
-        <v>0.5654</v>
+        <v>0.6098</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
@@ -7599,7 +7599,7 @@
         <v>1987</v>
       </c>
       <c r="X61" t="n">
-        <v>0.3857</v>
+        <v>0.1338</v>
       </c>
       <c r="Y61" t="inlineStr">
         <is>
@@ -7635,7 +7635,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>u m n+p</t>
+          <t>u m p</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -7647,16 +7647,16 @@
         <v>0.0001</v>
       </c>
       <c r="I62" t="n">
-        <v>0.3927</v>
+        <v>0.1047</v>
       </c>
       <c r="J62" t="n">
-        <v>0.046</v>
+        <v>0.156</v>
       </c>
       <c r="K62" t="n">
-        <v>0.3334</v>
+        <v>0.3021</v>
       </c>
       <c r="L62" t="n">
-        <v>2.2469</v>
+        <v>1.5226</v>
       </c>
       <c r="M62" t="n">
         <v>18</v>
@@ -7665,17 +7665,17 @@
         <v>17</v>
       </c>
       <c r="O62" t="n">
-        <v>0.1106</v>
+        <v>-0.1682</v>
       </c>
       <c r="P62" t="n">
-        <v>0.7204</v>
+        <v>0.3595</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.6098</v>
+        <v>0.5276999999999999</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>wrong_direction</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -7689,16 +7689,18 @@
         </is>
       </c>
       <c r="U62" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V62" t="n">
-        <v>5.8824</v>
-      </c>
-      <c r="W62" t="n">
-        <v>1987</v>
+        <v>17.6471</v>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>1987; 1988; 1989</t>
+        </is>
       </c>
       <c r="X62" t="n">
-        <v>0.1338</v>
+        <v>0.0597</v>
       </c>
       <c r="Y62" t="inlineStr">
         <is>
@@ -7734,7 +7736,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>u m p</t>
+          <t>u u n</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -7746,35 +7748,35 @@
         <v>0.0001</v>
       </c>
       <c r="I63" t="n">
-        <v>0.1047</v>
+        <v>0.1045</v>
       </c>
       <c r="J63" t="n">
-        <v>0.156</v>
+        <v>0.0883</v>
       </c>
       <c r="K63" t="n">
-        <v>0.3021</v>
+        <v>0.5848</v>
       </c>
       <c r="L63" t="n">
-        <v>1.5226</v>
+        <v>1.6611</v>
       </c>
       <c r="M63" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="N63" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="O63" t="n">
-        <v>-0.1682</v>
+        <v>0.2216</v>
       </c>
       <c r="P63" t="n">
-        <v>0.3595</v>
+        <v>0.3918</v>
       </c>
       <c r="Q63" t="n">
-        <v>0.5276999999999999</v>
+        <v>0.1702</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>wrong_direction</t>
+          <t>accurate</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -7788,18 +7790,18 @@
         </is>
       </c>
       <c r="U63" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="V63" t="n">
-        <v>17.6471</v>
+        <v>36.6667</v>
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>1987; 1988; 1989</t>
+          <t>1987; 1989; 1990; 1999; 2000; 2004; 2005; 2009; 2010; 2011; 2012</t>
         </is>
       </c>
       <c r="X63" t="n">
-        <v>0.0597</v>
+        <v>0.1747</v>
       </c>
       <c r="Y63" t="inlineStr">
         <is>
@@ -7835,28 +7837,28 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>u u n</t>
+          <t>u u n+p</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>increasing</t>
         </is>
       </c>
       <c r="H64" t="n">
         <v>0.0001</v>
       </c>
       <c r="I64" t="n">
-        <v>0.1045</v>
+        <v>0.0062</v>
       </c>
       <c r="J64" t="n">
-        <v>0.0883</v>
+        <v>0.231</v>
       </c>
       <c r="K64" t="n">
-        <v>0.5848</v>
+        <v>0.3003</v>
       </c>
       <c r="L64" t="n">
-        <v>1.6611</v>
+        <v>1.8544</v>
       </c>
       <c r="M64" t="n">
         <v>31</v>
@@ -7865,46 +7867,44 @@
         <v>30</v>
       </c>
       <c r="O64" t="n">
-        <v>0.2216</v>
+        <v>0.1074</v>
       </c>
       <c r="P64" t="n">
-        <v>0.3918</v>
+        <v>0.5688</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.1702</v>
+        <v>0.4614</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T64" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T64" t="n">
+        <v>4</v>
       </c>
       <c r="U64" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="V64" t="n">
-        <v>36.6667</v>
+        <v>10</v>
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>1987; 1989; 1990; 1999; 2000; 2004; 2005; 2009; 2010; 2011; 2012</t>
+          <t>1987; 1998; 1999</t>
         </is>
       </c>
       <c r="X64" t="n">
-        <v>0.1747</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="Y64" t="inlineStr">
         <is>
-          <t>non-directional</t>
+          <t>increasing</t>
         </is>
       </c>
     </row>
@@ -7936,28 +7936,28 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>u u n+p</t>
+          <t>u u p</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>0.0062</v>
+        <v>0.2916</v>
       </c>
       <c r="J65" t="n">
-        <v>0.231</v>
+        <v>0.0383</v>
       </c>
       <c r="K65" t="n">
-        <v>0.3003</v>
+        <v>0.2868</v>
       </c>
       <c r="L65" t="n">
-        <v>1.8544</v>
+        <v>1.1136</v>
       </c>
       <c r="M65" t="n">
         <v>31</v>
@@ -7966,76 +7966,78 @@
         <v>30</v>
       </c>
       <c r="O65" t="n">
-        <v>0.1074</v>
+        <v>0.123</v>
       </c>
       <c r="P65" t="n">
-        <v>0.5688</v>
+        <v>0.0737</v>
       </c>
       <c r="Q65" t="n">
-        <v>0.4614</v>
+        <v>-0.0494</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>accurate</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T65" t="n">
-        <v>4</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U65" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="V65" t="n">
-        <v>10</v>
+        <v>43.3333</v>
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>1987; 1998; 1999</t>
+          <t>1989; 1990; 1992; 1993; 1996; 2001; 2003; 2005; 2009; 2010; 2012; 2013; 2016</t>
         </is>
       </c>
       <c r="X65" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.6352</v>
       </c>
       <c r="Y65" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>KNZ</t>
+          <t>LUQ</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Konza Prairie</t>
+          <t>Luquillo</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Forest</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Fertilization</t>
+          <t>Vegetation Removal</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Flux</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>u u p</t>
+          <t>No trim + debris</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -8044,34 +8046,34 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>-0.0001</v>
       </c>
       <c r="I66" t="n">
-        <v>0.2916</v>
+        <v>0.4728</v>
       </c>
       <c r="J66" t="n">
-        <v>0.0383</v>
+        <v>0.1827</v>
       </c>
       <c r="K66" t="n">
-        <v>0.2868</v>
+        <v>0.0779</v>
       </c>
       <c r="L66" t="n">
-        <v>1.1136</v>
+        <v>1.1178</v>
       </c>
       <c r="M66" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="N66" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="O66" t="n">
-        <v>0.123</v>
+        <v>0.1151</v>
       </c>
       <c r="P66" t="n">
-        <v>0.0737</v>
+        <v>0.1089</v>
       </c>
       <c r="Q66" t="n">
-        <v>-0.0494</v>
+        <v>-0.0062</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
@@ -8089,18 +8091,18 @@
         </is>
       </c>
       <c r="U66" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="V66" t="n">
-        <v>43.3333</v>
+        <v>0</v>
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>1989; 1990; 1992; 1993; 1996; 2001; 2003; 2005; 2009; 2010; 2012; 2013; 2016</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="X66" t="n">
-        <v>0.6352</v>
+        <v>0.4618</v>
       </c>
       <c r="Y66" t="inlineStr">
         <is>
@@ -8136,7 +8138,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>No trim + debris</t>
+          <t>Trim &amp; clear</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -8145,19 +8147,19 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>-0.0001</v>
+        <v>0.0001</v>
       </c>
       <c r="I67" t="n">
-        <v>0.4728</v>
+        <v>0.3629</v>
       </c>
       <c r="J67" t="n">
-        <v>0.1827</v>
+        <v>0.2763</v>
       </c>
       <c r="K67" t="n">
-        <v>0.0779</v>
+        <v>0.1124</v>
       </c>
       <c r="L67" t="n">
-        <v>1.1178</v>
+        <v>0.9406</v>
       </c>
       <c r="M67" t="n">
         <v>5</v>
@@ -8166,13 +8168,13 @@
         <v>4</v>
       </c>
       <c r="O67" t="n">
-        <v>0.1151</v>
+        <v>-0.1101</v>
       </c>
       <c r="P67" t="n">
-        <v>0.1089</v>
+        <v>-0.06610000000000001</v>
       </c>
       <c r="Q67" t="n">
-        <v>-0.0062</v>
+        <v>0.044</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -8190,18 +8192,18 @@
         </is>
       </c>
       <c r="U67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V67" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>2008; 2009</t>
         </is>
       </c>
       <c r="X67" t="n">
-        <v>0.4618</v>
+        <v>0.3508</v>
       </c>
       <c r="Y67" t="inlineStr">
         <is>
@@ -8237,7 +8239,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Trim &amp; clear</t>
+          <t>Trim + debris</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -8246,19 +8248,19 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0.3629</v>
+        <v>0.8642</v>
       </c>
       <c r="J68" t="n">
-        <v>0.2763</v>
+        <v>0.0114</v>
       </c>
       <c r="K68" t="n">
-        <v>0.1124</v>
+        <v>0.0954</v>
       </c>
       <c r="L68" t="n">
-        <v>0.9406</v>
+        <v>0.975</v>
       </c>
       <c r="M68" t="n">
         <v>5</v>
@@ -8267,13 +8269,13 @@
         <v>4</v>
       </c>
       <c r="O68" t="n">
-        <v>-0.1101</v>
+        <v>-0.0232</v>
       </c>
       <c r="P68" t="n">
-        <v>-0.06610000000000001</v>
+        <v>-0.029</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.044</v>
+        <v>-0.0058</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -8298,11 +8300,11 @@
       </c>
       <c r="W68" t="inlineStr">
         <is>
-          <t>2008; 2009</t>
+          <t>2007; 2008</t>
         </is>
       </c>
       <c r="X68" t="n">
-        <v>0.3508</v>
+        <v>0.8448</v>
       </c>
       <c r="Y68" t="inlineStr">
         <is>
@@ -8313,22 +8315,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LUQ</t>
+          <t>MCM</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Luquillo</t>
+          <t>McMurdo Dry Valleys</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Tundra</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Vegetation Removal</t>
+          <t>Fertilization</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -8338,47 +8340,47 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Trim + debris</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="I69" t="n">
-        <v>0.8642</v>
+        <v>0.4514</v>
       </c>
       <c r="J69" t="n">
-        <v>0.0114</v>
+        <v>0.199</v>
       </c>
       <c r="K69" t="n">
-        <v>0.0954</v>
+        <v>0.6064000000000001</v>
       </c>
       <c r="L69" t="n">
-        <v>0.975</v>
+        <v>1.9005</v>
       </c>
       <c r="M69" t="n">
         <v>5</v>
       </c>
       <c r="N69" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O69" t="n">
-        <v>-0.0232</v>
+        <v>0.1083</v>
       </c>
       <c r="P69" t="n">
-        <v>-0.029</v>
+        <v>0.4546</v>
       </c>
       <c r="Q69" t="n">
-        <v>-0.0058</v>
+        <v>0.3464</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
@@ -8392,18 +8394,18 @@
         </is>
       </c>
       <c r="U69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V69" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>2007; 2008</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="X69" t="n">
-        <v>0.8448</v>
+        <v>0.3521</v>
       </c>
       <c r="Y69" t="inlineStr">
         <is>
@@ -8439,28 +8441,28 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H70" t="n">
-        <v>0.0002</v>
+        <v>0.0009</v>
       </c>
       <c r="I70" t="n">
-        <v>0.0486</v>
+        <v>0.2537</v>
       </c>
       <c r="J70" t="n">
-        <v>0.7756999999999999</v>
+        <v>0.3981</v>
       </c>
       <c r="K70" t="n">
-        <v>0.1389</v>
+        <v>0.5974</v>
       </c>
       <c r="L70" t="n">
-        <v>1.4399</v>
+        <v>2.3192</v>
       </c>
       <c r="M70" t="n">
         <v>5</v>
@@ -8469,13 +8471,13 @@
         <v>7</v>
       </c>
       <c r="O70" t="n">
-        <v>0.1083</v>
+        <v>0.2283</v>
       </c>
       <c r="P70" t="n">
-        <v>0.3561</v>
+        <v>0.616</v>
       </c>
       <c r="Q70" t="n">
-        <v>0.2478</v>
+        <v>0.3876</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
@@ -8484,11 +8486,13 @@
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T70" t="n">
-        <v>6.0014</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U70" t="n">
         <v>0</v>
@@ -8502,11 +8506,11 @@
         </is>
       </c>
       <c r="X70" t="n">
-        <v>0.0405</v>
+        <v>0.1737</v>
       </c>
       <c r="Y70" t="inlineStr">
         <is>
-          <t>increasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
@@ -8538,7 +8542,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>CP</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -8547,19 +8551,19 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>0.0005</v>
+        <v>0.0009</v>
       </c>
       <c r="I71" t="n">
-        <v>0.1773</v>
+        <v>0.4259</v>
       </c>
       <c r="J71" t="n">
-        <v>0.507</v>
+        <v>0.2197</v>
       </c>
       <c r="K71" t="n">
-        <v>0.3852</v>
+        <v>0.9553</v>
       </c>
       <c r="L71" t="n">
-        <v>1.7735</v>
+        <v>1.9132</v>
       </c>
       <c r="M71" t="n">
         <v>5</v>
@@ -8568,17 +8572,17 @@
         <v>7</v>
       </c>
       <c r="O71" t="n">
-        <v>0.2283</v>
+        <v>-0.6972</v>
       </c>
       <c r="P71" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.2441</v>
       </c>
       <c r="Q71" t="n">
-        <v>0.2914</v>
+        <v>0.9412</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>wrong_direction</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
@@ -8592,18 +8596,16 @@
         </is>
       </c>
       <c r="U71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V71" t="n">
-        <v>0</v>
-      </c>
-      <c r="W71" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="W71" t="n">
+        <v>2007</v>
       </c>
       <c r="X71" t="n">
-        <v>0.1502</v>
+        <v>0.2169</v>
       </c>
       <c r="Y71" t="inlineStr">
         <is>
@@ -8639,7 +8641,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>CP</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -8648,19 +8650,19 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="I72" t="n">
-        <v>0.1635</v>
+        <v>0.3365</v>
       </c>
       <c r="J72" t="n">
-        <v>0.5294</v>
+        <v>0.3029</v>
       </c>
       <c r="K72" t="n">
-        <v>0.3917</v>
+        <v>0.4383</v>
       </c>
       <c r="L72" t="n">
-        <v>1.232</v>
+        <v>1.256</v>
       </c>
       <c r="M72" t="n">
         <v>5</v>
@@ -8669,26 +8671,28 @@
         <v>7</v>
       </c>
       <c r="O72" t="n">
-        <v>-0.6972</v>
+        <v>-0.4774</v>
       </c>
       <c r="P72" t="n">
-        <v>0.1251</v>
+        <v>0.09760000000000001</v>
       </c>
       <c r="Q72" t="n">
-        <v>0.8223</v>
+        <v>0.5750999999999999</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>wrong_direction</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T72" t="n">
-        <v>6.0014</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U72" t="n">
         <v>1</v>
@@ -8700,7 +8704,7 @@
         <v>2007</v>
       </c>
       <c r="X72" t="n">
-        <v>0.1016</v>
+        <v>0.2304</v>
       </c>
       <c r="Y72" t="inlineStr">
         <is>
@@ -8736,28 +8740,28 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>0.0002</v>
+        <v>0.0003</v>
       </c>
       <c r="I73" t="n">
-        <v>0.3808</v>
+        <v>0.3513</v>
       </c>
       <c r="J73" t="n">
-        <v>0.2594</v>
+        <v>0.2878</v>
       </c>
       <c r="K73" t="n">
-        <v>0.2944</v>
+        <v>0.4071</v>
       </c>
       <c r="L73" t="n">
-        <v>1.057</v>
+        <v>1.2386</v>
       </c>
       <c r="M73" t="n">
         <v>5</v>
@@ -8766,17 +8770,17 @@
         <v>7</v>
       </c>
       <c r="O73" t="n">
-        <v>-0.4774</v>
+        <v>-0.263</v>
       </c>
       <c r="P73" t="n">
-        <v>0.0176</v>
+        <v>0.1238</v>
       </c>
       <c r="Q73" t="n">
-        <v>0.495</v>
+        <v>0.3868</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>wrong_direction</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
@@ -8799,7 +8803,7 @@
         <v>2007</v>
       </c>
       <c r="X73" t="n">
-        <v>0.2481</v>
+        <v>0.2585</v>
       </c>
       <c r="Y73" t="inlineStr">
         <is>
@@ -8810,17 +8814,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>MCM</t>
+          <t>NTL</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>McMurdo Dry Valleys</t>
+          <t>North Temperate Lakes</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Tundra</t>
+          <t>Freshwater</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8830,73 +8834,77 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Flux</t>
+          <t>Proxy</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>added</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H74" t="n">
-        <v>0.0001</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="I74" t="n">
-        <v>0.1682</v>
+        <v>0.602</v>
       </c>
       <c r="J74" t="n">
-        <v>0.5217000000000001</v>
+        <v>0.1584</v>
       </c>
       <c r="K74" t="n">
-        <v>0.1758</v>
+        <v>0.3554</v>
       </c>
       <c r="L74" t="n">
-        <v>1.0571</v>
+        <v>3.9423</v>
       </c>
       <c r="M74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O74" t="n">
-        <v>-0.263</v>
+        <v>1.4546</v>
       </c>
       <c r="P74" t="n">
-        <v>0.0419</v>
+        <v>1.3257</v>
       </c>
       <c r="Q74" t="n">
-        <v>0.3049</v>
+        <v>-0.1289</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>underestimate</t>
+          <t>accurate</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T74" t="n">
-        <v>6.0014</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V74" t="n">
-        <v>25</v>
-      </c>
-      <c r="W74" t="n">
-        <v>2007</v>
+        <v>0</v>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="X74" t="n">
-        <v>0.1397</v>
+        <v>0.5039</v>
       </c>
       <c r="Y74" t="inlineStr">
         <is>
@@ -8907,17 +8915,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>NTL</t>
+          <t>NWT</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>North Temperate Lakes</t>
+          <t>Niwot Ridge</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Freshwater</t>
+          <t>Tundra</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8927,77 +8935,75 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Proxy</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>added</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H75" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>0.602</v>
+        <v>0.7449</v>
       </c>
       <c r="J75" t="n">
-        <v>0.1584</v>
+        <v>0.0111</v>
       </c>
       <c r="K75" t="n">
-        <v>0.3554</v>
+        <v>0.1307</v>
       </c>
       <c r="L75" t="n">
-        <v>3.9423</v>
+        <v>0.9866</v>
       </c>
       <c r="M75" t="n">
+        <v>12</v>
+      </c>
+      <c r="N75" t="n">
+        <v>12</v>
+      </c>
+      <c r="O75" t="n">
+        <v>-0.0572</v>
+      </c>
+      <c r="P75" t="n">
+        <v>-0.021</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0.0362</v>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T75" t="n">
         <v>4</v>
       </c>
-      <c r="N75" t="n">
-        <v>6</v>
-      </c>
-      <c r="O75" t="n">
-        <v>1.4546</v>
-      </c>
-      <c r="P75" t="n">
-        <v>1.3257</v>
-      </c>
-      <c r="Q75" t="n">
-        <v>-0.1289</v>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>accurate</t>
-        </is>
-      </c>
-      <c r="S75" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T75" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="U75" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="V75" t="n">
-        <v>0</v>
+        <v>72.7273</v>
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>2008; 2009; 2010; 2012; 2014; 2015; 2017; 2019</t>
         </is>
       </c>
       <c r="X75" t="n">
-        <v>0.5039</v>
+        <v>0.7216</v>
       </c>
       <c r="Y75" t="inlineStr">
         <is>
@@ -9008,17 +9014,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>NWT</t>
+          <t>PIE</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Niwot Ridge</t>
+          <t>Plum Island Ecosystems</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Tundra</t>
+          <t>Coastal</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -9028,12 +9034,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Proxy</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Enriched</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -9045,31 +9051,31 @@
         <v>0</v>
       </c>
       <c r="I76" t="n">
-        <v>0.7449</v>
+        <v>0.7993</v>
       </c>
       <c r="J76" t="n">
-        <v>0.0111</v>
+        <v>0.0048</v>
       </c>
       <c r="K76" t="n">
-        <v>0.1307</v>
+        <v>0.1081</v>
       </c>
       <c r="L76" t="n">
-        <v>0.9866</v>
+        <v>1.1473</v>
       </c>
       <c r="M76" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="N76" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="O76" t="n">
-        <v>-0.0572</v>
+        <v>0.078</v>
       </c>
       <c r="P76" t="n">
-        <v>-0.021</v>
+        <v>0.1324</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.0362</v>
+        <v>0.0544</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
@@ -9078,25 +9084,27 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T76" t="n">
-        <v>4</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U76" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="V76" t="n">
-        <v>72.7273</v>
+        <v>0</v>
       </c>
       <c r="W76" t="inlineStr">
         <is>
-          <t>2008; 2009; 2010; 2012; 2014; 2015; 2017; 2019</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="X76" t="n">
-        <v>0.7216</v>
+        <v>0.7892</v>
       </c>
       <c r="Y76" t="inlineStr">
         <is>
@@ -9107,12 +9115,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PIE</t>
+          <t>SBC</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Plum Island Ecosystems</t>
+          <t>Santa Barbara Coastal</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -9122,38 +9130,38 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Fertilization</t>
+          <t>Vegetation Removal</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Proxy</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Enriched</t>
+          <t>ANNUAL</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>decreasing</t>
         </is>
       </c>
       <c r="H77" t="n">
         <v>0</v>
       </c>
       <c r="I77" t="n">
-        <v>0.7993</v>
+        <v>0.0171</v>
       </c>
       <c r="J77" t="n">
-        <v>0.0048</v>
+        <v>0.3434</v>
       </c>
       <c r="K77" t="n">
-        <v>0.1081</v>
+        <v>0.1635</v>
       </c>
       <c r="L77" t="n">
-        <v>1.1473</v>
+        <v>0.8928</v>
       </c>
       <c r="M77" t="n">
         <v>16</v>
@@ -9162,46 +9170,44 @@
         <v>15</v>
       </c>
       <c r="O77" t="n">
-        <v>0.078</v>
+        <v>0.0166</v>
       </c>
       <c r="P77" t="n">
-        <v>0.1324</v>
+        <v>-0.227</v>
       </c>
       <c r="Q77" t="n">
-        <v>0.0544</v>
+        <v>-0.2435</v>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>overestimate</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T77" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T77" t="n">
+        <v>4</v>
       </c>
       <c r="U77" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="V77" t="n">
-        <v>0</v>
+        <v>33.3333</v>
       </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>2010; 2015; 2016; 2018; 2019</t>
         </is>
       </c>
       <c r="X77" t="n">
-        <v>0.7892</v>
+        <v>0.0163</v>
       </c>
       <c r="Y77" t="inlineStr">
         <is>
-          <t>non-directional</t>
+          <t>decreasing</t>
         </is>
       </c>
     </row>
@@ -9233,94 +9239,98 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>ANNUAL</t>
+          <t>CONTINUAL</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>decreasing</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="H78" t="n">
-        <v>0</v>
+        <v>-0.0001</v>
       </c>
       <c r="I78" t="n">
-        <v>0.0163</v>
+        <v>0.1913</v>
       </c>
       <c r="J78" t="n">
-        <v>0.3472</v>
+        <v>0.1378</v>
       </c>
       <c r="K78" t="n">
-        <v>0.1888</v>
+        <v>0.1778</v>
       </c>
       <c r="L78" t="n">
-        <v>0.748</v>
+        <v>1.5176</v>
       </c>
       <c r="M78" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="N78" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O78" t="n">
-        <v>-0.0567</v>
+        <v>0.237</v>
       </c>
       <c r="P78" t="n">
-        <v>-0.3059</v>
+        <v>0.2897</v>
       </c>
       <c r="Q78" t="n">
-        <v>-0.2492</v>
+        <v>0.0527</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>overestimate</t>
+          <t>accurate</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T78" t="n">
-        <v>6.0014</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V78" t="n">
-        <v>6.6667</v>
-      </c>
-      <c r="W78" t="n">
-        <v>2009</v>
+        <v>0</v>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="X78" t="n">
-        <v>0.0169</v>
+        <v>0.1495</v>
       </c>
       <c r="Y78" t="inlineStr">
         <is>
-          <t>decreasing</t>
+          <t>non-directional</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SBC</t>
+          <t>SEV</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Santa Barbara Coastal</t>
+          <t>Sevilleta</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Coastal</t>
+          <t>Grassland</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Vegetation Removal</t>
+          <t>Fertilization</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -9330,7 +9340,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>CONTINUAL</t>
+          <t>F</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -9342,31 +9352,31 @@
         <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>0.2214</v>
+        <v>0.3227</v>
       </c>
       <c r="J79" t="n">
-        <v>0.1218</v>
+        <v>0.0543</v>
       </c>
       <c r="K79" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.2687</v>
       </c>
       <c r="L79" t="n">
-        <v>0.9978</v>
+        <v>1.2023</v>
       </c>
       <c r="M79" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="N79" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="O79" t="n">
-        <v>0.066</v>
+        <v>0.2175</v>
       </c>
       <c r="P79" t="n">
-        <v>-0.0066</v>
+        <v>0.1507</v>
       </c>
       <c r="Q79" t="n">
-        <v>-0.0727</v>
+        <v>-0.0668</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
@@ -9375,25 +9385,27 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T79" t="n">
-        <v>7.0007</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="U79" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V79" t="n">
-        <v>38.4615</v>
+        <v>15.7895</v>
       </c>
       <c r="W79" t="inlineStr">
         <is>
-          <t>2011; 2012; 2014; 2018; 2020</t>
+          <t>2006; 2018; 2022</t>
         </is>
       </c>
       <c r="X79" t="n">
-        <v>0.2619</v>
+        <v>0.2347</v>
       </c>
       <c r="Y79" t="inlineStr">
         <is>
@@ -9404,22 +9416,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SEV</t>
+          <t>VCR</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Sevilleta</t>
+          <t>Virginia Coast Reserve</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Coastal</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Fertilization</t>
+          <t>Disturbance</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -9429,47 +9441,47 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Wrack</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>stable</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="H80" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="I80" t="n">
-        <v>0.3227</v>
+        <v>0.0877</v>
       </c>
       <c r="J80" t="n">
-        <v>0.0543</v>
+        <v>0.6756</v>
       </c>
       <c r="K80" t="n">
-        <v>0.2687</v>
+        <v>0.4931</v>
       </c>
       <c r="L80" t="n">
-        <v>1.2023</v>
+        <v>0.7156</v>
       </c>
       <c r="M80" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="N80" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="O80" t="n">
-        <v>0.2175</v>
+        <v>-0.8652</v>
       </c>
       <c r="P80" t="n">
-        <v>0.1507</v>
+        <v>-0.55</v>
       </c>
       <c r="Q80" t="n">
-        <v>-0.0668</v>
+        <v>0.3153</v>
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
@@ -9483,121 +9495,20 @@
         </is>
       </c>
       <c r="U80" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V80" t="n">
-        <v>15.7895</v>
+        <v>0</v>
       </c>
       <c r="W80" t="inlineStr">
         <is>
-          <t>2006; 2018; 2022</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="X80" t="n">
-        <v>0.2347</v>
+        <v>0.1234</v>
       </c>
       <c r="Y80" t="inlineStr">
-        <is>
-          <t>non-directional</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>VCR</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Virginia Coast Reserve</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Coastal</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Disturbance</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Wrack</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
-      <c r="H81" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="I81" t="n">
-        <v>0.0877</v>
-      </c>
-      <c r="J81" t="n">
-        <v>0.6756</v>
-      </c>
-      <c r="K81" t="n">
-        <v>0.4931</v>
-      </c>
-      <c r="L81" t="n">
-        <v>0.7156</v>
-      </c>
-      <c r="M81" t="n">
-        <v>5</v>
-      </c>
-      <c r="N81" t="n">
-        <v>4</v>
-      </c>
-      <c r="O81" t="n">
-        <v>-0.8652</v>
-      </c>
-      <c r="P81" t="n">
-        <v>-0.55</v>
-      </c>
-      <c r="Q81" t="n">
-        <v>0.3153</v>
-      </c>
-      <c r="R81" t="inlineStr">
-        <is>
-          <t>underestimate</t>
-        </is>
-      </c>
-      <c r="S81" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T81" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="U81" t="n">
-        <v>0</v>
-      </c>
-      <c r="V81" t="n">
-        <v>0</v>
-      </c>
-      <c r="W81" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="X81" t="n">
-        <v>0.1234</v>
-      </c>
-      <c r="Y81" t="inlineStr">
         <is>
           <t>non-directional</t>
         </is>
@@ -9614,7 +9525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11200,23 +11111,21 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2012</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>0.192047; -0.01479</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>0.0754; 0.0173</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>0.115298</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.0187</v>
       </c>
       <c r="J39" t="n">
         <v>5</v>
@@ -11255,10 +11164,10 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0.005282</v>
+        <v>0.012176</v>
       </c>
       <c r="I40" t="n">
-        <v>0.4198</v>
+        <v>0.367</v>
       </c>
       <c r="J40" t="n">
         <v>5</v>
@@ -11297,7 +11206,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.013621</v>
+        <v>0.013761</v>
       </c>
       <c r="I41" t="n">
         <v>0.0001</v>
@@ -11338,12 +11247,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>NA; 0.010853</t>
+          <t>NA; 0.011344</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>NA; 0.014</t>
+          <t>NA; 0.0129</t>
         </is>
       </c>
       <c r="J42" t="n">
@@ -11383,10 +11292,10 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0.003714</v>
+        <v>0.002812</v>
       </c>
       <c r="I43" t="n">
-        <v>0.1166</v>
+        <v>0.2115</v>
       </c>
       <c r="J43" t="n">
         <v>5</v>
@@ -11471,10 +11380,10 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>0.014312</v>
+        <v>0.00661</v>
       </c>
       <c r="I45" t="n">
-        <v>0.2938</v>
+        <v>0.468</v>
       </c>
       <c r="J45" t="n">
         <v>5</v>
@@ -11513,10 +11422,10 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>0.020858</v>
+        <v>0.011057</v>
       </c>
       <c r="I46" t="n">
-        <v>0.1221</v>
+        <v>0.2603</v>
       </c>
       <c r="J46" t="n">
         <v>5</v>
@@ -11551,17 +11460,17 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2005; 2011</t>
+          <t>2005; 2010</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>0.005958; 0.139268; 0.050223</t>
+          <t>0.001956; 0.077894; 0.006294</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>0.7821; 0.023; 0.6818</t>
+          <t>0.8832; 0.2338; 0.9093</t>
         </is>
       </c>
       <c r="J47" t="n">
@@ -11571,12 +11480,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>KBS</t>
+          <t>KNZ</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Kellogg Biological Station</t>
+          <t>Konza Prairie</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -11586,11 +11495,11 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>T6</t>
+          <t>b m c</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -11601,10 +11510,10 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>0.022589</v>
+        <v>0.032832</v>
       </c>
       <c r="I48" t="n">
-        <v>0.4387</v>
+        <v>0.1116</v>
       </c>
       <c r="J48" t="n">
         <v>5</v>
@@ -11628,25 +11537,27 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>b m c</t>
+          <t>b m n</t>
         </is>
       </c>
       <c r="E49" t="n">
         <v>18</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H49" t="n">
-        <v>0.032832</v>
-      </c>
-      <c r="I49" t="n">
-        <v>0.1116</v>
+        <v>1</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1994</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>0.160072; 0.075375</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>0.1974; 0.3537</t>
+        </is>
       </c>
       <c r="J49" t="n">
         <v>5</v>
@@ -11670,27 +11581,25 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>b m n</t>
+          <t>b m n+p</t>
         </is>
       </c>
       <c r="E50" t="n">
         <v>18</v>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" t="n">
-        <v>1994</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>0.160072; 0.075375</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>0.1974; 0.3537</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>0.064554</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.0819</v>
       </c>
       <c r="J50" t="n">
         <v>5</v>
@@ -11714,25 +11623,29 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>b m n+p</t>
+          <t>b m p</t>
         </is>
       </c>
       <c r="E51" t="n">
         <v>18</v>
       </c>
       <c r="F51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H51" t="n">
-        <v>0.064554</v>
-      </c>
-      <c r="I51" t="n">
-        <v>0.0819</v>
+          <t>1993; 1995</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>0.071759; 0.169856; -0.013081</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>0.388; NaN; 0.8032</t>
+        </is>
       </c>
       <c r="J51" t="n">
         <v>5</v>
@@ -11756,28 +11669,26 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>b m p</t>
+          <t>b u c</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F52" t="n">
-        <v>2</v>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>1993; 1995</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1999</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>0.071759; 0.169856; -0.013081</t>
+          <t>-0.018375; 0.650037</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>0.388; NaN; 0.8032</t>
+          <t>0.4411; 1e-04</t>
         </is>
       </c>
       <c r="J52" t="n">
@@ -11802,26 +11713,28 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>b u c</t>
+          <t>b u n</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" t="n">
-        <v>1999</v>
+        <v>2</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>1991; 1999</t>
+        </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>-0.018375; 0.650037</t>
+          <t>0.236309; -0.145587; 0.734654</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>0.4411; 1e-04</t>
+          <t>0.23; 0.2361; 2e-04</t>
         </is>
       </c>
       <c r="J53" t="n">
@@ -11846,7 +11759,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>b u n</t>
+          <t>b u n+p</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -11857,17 +11770,17 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>1991; 1999</t>
+          <t>1988; 2000</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>0.236309; -0.145587; 0.734654</t>
+          <t>0.255589; -0.059132; 0.762911</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>0.23; 0.2361; 2e-04</t>
+          <t>0.8568; 0.4876; 0</t>
         </is>
       </c>
       <c r="J54" t="n">
@@ -11892,28 +11805,26 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>b u n+p</t>
+          <t>b u p</t>
         </is>
       </c>
       <c r="E55" t="n">
         <v>31</v>
       </c>
       <c r="F55" t="n">
-        <v>2</v>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>1988; 2000</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1997</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>0.255589; -0.059132; 0.762911</t>
+          <t>-0.000102; 0.253901</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>0.8568; 0.4876; 0</t>
+          <t>0.9978; 0</t>
         </is>
       </c>
       <c r="J55" t="n">
@@ -11938,27 +11849,25 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>b u p</t>
+          <t>u m c</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F56" t="n">
-        <v>1</v>
-      </c>
-      <c r="G56" t="n">
-        <v>1997</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>-0.000102; 0.253901</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>0.9978; 0</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>0.01558</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0.4047</v>
       </c>
       <c r="J56" t="n">
         <v>5</v>
@@ -11982,7 +11891,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>u m c</t>
+          <t>u m n</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -11997,10 +11906,10 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>0.01558</v>
+        <v>0.002029</v>
       </c>
       <c r="I57" t="n">
-        <v>0.4047</v>
+        <v>0.9584</v>
       </c>
       <c r="J57" t="n">
         <v>5</v>
@@ -12024,7 +11933,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>u m n</t>
+          <t>u m n+p</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -12039,10 +11948,10 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>0.002029</v>
+        <v>0.030098</v>
       </c>
       <c r="I58" t="n">
-        <v>0.9584</v>
+        <v>0.3927</v>
       </c>
       <c r="J58" t="n">
         <v>5</v>
@@ -12066,7 +11975,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>u m n+p</t>
+          <t>u m p</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -12081,10 +11990,10 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>0.030098</v>
+        <v>0.034035</v>
       </c>
       <c r="I59" t="n">
-        <v>0.3927</v>
+        <v>0.1047</v>
       </c>
       <c r="J59" t="n">
         <v>5</v>
@@ -12108,11 +12017,11 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>u m p</t>
+          <t>u u n</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -12123,10 +12032,10 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>0.034035</v>
+        <v>0.031744</v>
       </c>
       <c r="I60" t="n">
-        <v>0.1047</v>
+        <v>0.1045</v>
       </c>
       <c r="J60" t="n">
         <v>5</v>
@@ -12150,25 +12059,27 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>u u n</t>
+          <t>u u n+p</t>
         </is>
       </c>
       <c r="E61" t="n">
         <v>31</v>
       </c>
       <c r="F61" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H61" t="n">
-        <v>0.031744</v>
-      </c>
-      <c r="I61" t="n">
-        <v>0.1045</v>
+        <v>1</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2010</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>0.017828; 0.133762</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>0.2345; 0.0937</t>
+        </is>
       </c>
       <c r="J61" t="n">
         <v>5</v>
@@ -12192,27 +12103,25 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>u u n+p</t>
+          <t>u u p</t>
         </is>
       </c>
       <c r="E62" t="n">
         <v>31</v>
       </c>
       <c r="F62" t="n">
-        <v>1</v>
-      </c>
-      <c r="G62" t="n">
-        <v>2010</v>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>0.017828; 0.133762</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>0.2345; 0.0937</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>0.006871</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0.2916</v>
       </c>
       <c r="J62" t="n">
         <v>5</v>
@@ -12221,26 +12130,26 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>KNZ</t>
+          <t>LUQ</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Konza Prairie</t>
+          <t>Luquillo</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Forest</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>u u p</t>
+          <t>No trim + debris</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
@@ -12251,10 +12160,10 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>0.006871</v>
+        <v>-0.023518</v>
       </c>
       <c r="I63" t="n">
-        <v>0.2916</v>
+        <v>0.4731</v>
       </c>
       <c r="J63" t="n">
         <v>5</v>
@@ -12278,7 +12187,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>No trim + debris</t>
+          <t>Trim &amp; clear</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -12293,10 +12202,10 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>-0.023518</v>
+        <v>0.035192</v>
       </c>
       <c r="I64" t="n">
-        <v>0.4731</v>
+        <v>0.3625</v>
       </c>
       <c r="J64" t="n">
         <v>5</v>
@@ -12320,7 +12229,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Trim &amp; clear</t>
+          <t>Trim + debris</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -12335,10 +12244,10 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0.035192</v>
+        <v>0.006295</v>
       </c>
       <c r="I65" t="n">
-        <v>0.3625</v>
+        <v>0.8641</v>
       </c>
       <c r="J65" t="n">
         <v>5</v>
@@ -12347,22 +12256,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LUQ</t>
+          <t>MCM</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Luquillo</t>
+          <t>McMurdo Dry Valleys</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Forest</t>
+          <t>Tundra</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Trim + debris</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -12377,10 +12286,10 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>0.006295</v>
+        <v>0.190221</v>
       </c>
       <c r="I66" t="n">
-        <v>0.8641</v>
+        <v>0.4516</v>
       </c>
       <c r="J66" t="n">
         <v>5</v>
@@ -12404,7 +12313,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -12419,10 +12328,10 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>0.065193</v>
+        <v>0.323469</v>
       </c>
       <c r="I67" t="n">
-        <v>0.0485</v>
+        <v>0.2538</v>
       </c>
       <c r="J67" t="n">
         <v>5</v>
@@ -12446,7 +12355,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>CP</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -12461,10 +12370,10 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>0.180051</v>
+        <v>0.316942</v>
       </c>
       <c r="I68" t="n">
-        <v>0.1772</v>
+        <v>0.426</v>
       </c>
       <c r="J68" t="n">
         <v>5</v>
@@ -12488,7 +12397,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>CP</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -12503,10 +12412,10 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>0.129964</v>
+        <v>0.112114</v>
       </c>
       <c r="I69" t="n">
-        <v>0.1635</v>
+        <v>0.3366</v>
       </c>
       <c r="J69" t="n">
         <v>5</v>
@@ -12530,7 +12439,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -12545,10 +12454,10 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>0.058661</v>
+        <v>0.100083</v>
       </c>
       <c r="I70" t="n">
-        <v>0.3807</v>
+        <v>0.3515</v>
       </c>
       <c r="J70" t="n">
         <v>5</v>
@@ -12557,12 +12466,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MCM</t>
+          <t>NWT</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>McMurdo Dry Valleys</t>
+          <t>Niwot Ridge</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -12572,11 +12481,11 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
@@ -12587,10 +12496,10 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>0.049677</v>
+        <v>-0.003616</v>
       </c>
       <c r="I71" t="n">
-        <v>0.1681</v>
+        <v>0.7448</v>
       </c>
       <c r="J71" t="n">
         <v>5</v>
@@ -12599,26 +12508,26 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>NWT</t>
+          <t>PIE</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Niwot Ridge</t>
+          <t>Plum Island Ecosystems</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Tundra</t>
+          <t>Coastal</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Enriched</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
@@ -12629,10 +12538,10 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>-0.003616</v>
+        <v>0.001802</v>
       </c>
       <c r="I72" t="n">
-        <v>0.7448</v>
+        <v>0.7991</v>
       </c>
       <c r="J72" t="n">
         <v>5</v>
@@ -12641,12 +12550,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PIE</t>
+          <t>SBC</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Plum Island Ecosystems</t>
+          <t>Santa Barbara Coastal</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -12656,25 +12565,29 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Enriched</t>
+          <t>ANNUAL</t>
         </is>
       </c>
       <c r="E73" t="n">
         <v>16</v>
       </c>
       <c r="F73" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H73" t="n">
-        <v>0.001802</v>
-      </c>
-      <c r="I73" t="n">
-        <v>0.7991</v>
+          <t>2009; 2022</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>0.01494; -0.006949; NA</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>NaN; 0.4482; NA</t>
+        </is>
       </c>
       <c r="J73" t="n">
         <v>5</v>
@@ -12698,26 +12611,26 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>ANNUAL</t>
+          <t>CONTINUAL</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F74" t="n">
         <v>1</v>
       </c>
       <c r="G74" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>-0.056052; -0.005063</t>
+          <t>0.0143; 0.054766</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>0.0462; 0.7255</t>
+          <t>0.5245; 0.6481</t>
         </is>
       </c>
       <c r="J74" t="n">
@@ -12727,26 +12640,26 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SBC</t>
+          <t>SEV</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Santa Barbara Coastal</t>
+          <t>Sevilleta</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Coastal</t>
+          <t>Grassland</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>CONTINUAL</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
@@ -12757,10 +12670,10 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>-0.008168999999999999</v>
+        <v>-0.012726</v>
       </c>
       <c r="I75" t="n">
-        <v>0.2214</v>
+        <v>0.3227</v>
       </c>
       <c r="J75" t="n">
         <v>5</v>
@@ -12769,26 +12682,26 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SEV</t>
+          <t>VCR</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Sevilleta</t>
+          <t>Virginia Coast Reserve</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Coastal</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Wrack</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
@@ -12799,54 +12712,12 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>-0.012726</v>
+        <v>0.183471</v>
       </c>
       <c r="I76" t="n">
-        <v>0.3227</v>
+        <v>0.0876</v>
       </c>
       <c r="J76" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>VCR</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Virginia Coast Reserve</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Coastal</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Wrack</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>5</v>
-      </c>
-      <c r="F77" t="n">
-        <v>0</v>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="H77" t="n">
-        <v>0.183471</v>
-      </c>
-      <c r="I77" t="n">
-        <v>0.0876</v>
-      </c>
-      <c r="J77" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Early-vs-full tolerance defined as a 20% difference between response ratios (ln 1.2)
Matches the wording used in the text ('differed by more than 20%'); the
sensitivity sweep and Fig. S1 are now expressed in percent. 46 accurate,
17 under, 7 over, 7 reversed (40% mispredicted).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -1694,7 +1694,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table S2. Per-treatment statistics for the 78 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; tolerance 0.2), years to first detection of a significant trend (directional treatments only), the number, percentage (of consecutive measurement transitions), and years of sign flips, and the P-value and directional call when the trend analysis is repeated on the log response ratio.</t>
+          <t>Table S2. Per-treatment statistics for the 78 classified treatment-experiment combinations: trend class, slope, P-value and R-squared of the linear fit of the response ratio over time, coefficient of variation (CV), mean response ratio, number of timepoints, record length, early (first three calendar years) and full-duration log response ratios (LRR) with their difference and classification (accurate, underestimate, overestimate, wrong direction; early and full-record response ratios within 20%), years to first detection of a significant trend (directional treatments only), the number, percentage (of consecutive measurement transitions), and years of sign flips, and the P-value and directional call when the trend analysis is repeated on the log response ratio.</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>underestimate</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>overestimate</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>accurate</t>
+          <t>overestimate</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">

</xml_diff>

<commit_message>
Per-site processing notes in site metadata, Table S1 and a Supplementary Methods section
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/supplement/Supplementary_Tables_S1-S3.xlsx
+++ b/docs/supplement/Supplementary_Tables_S1-S3.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -437,13 +437,14 @@
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table S1. Details of the 18 case-study datasets: setting, experiment, manipulation, response variable and type, years analyzed, number of years sampled, number of analyzable treatments (in parentheses, the number screened), EDI data-package identifier, and data citation.</t>
+          <t>Table S1. Details of the 18 case-study datasets: setting, experiment, manipulation, response variable and type, years analyzed, number of years sampled, number of analyzable treatments (in parentheses, the number screened), EDI data-package identifier, data citation, and dataset-specific processing notes (also given in the Supplementary Methods).</t>
         </is>
       </c>
     </row>
@@ -510,6 +511,11 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
+          <t>Processing Notes</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
           <t>Data Citation</t>
         </is>
       </c>
@@ -573,6 +579,11 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>Vegetation cover (carbon proxy) in disturbed vs. control plots. Monitoring of a marsh stopped once its disturbed plots had recovered, so after 2014 only the slowest sites remain; the balanced panel of all 12 sites (2010-2014) was analyzed.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>Pennings, S. C. (2022). Data from: “Critical slowing down: vegetation height, cover and composition assess resilience of tidal fresh, brackish and salt marshes following experimental disturbance at twelve sites across the estuarine landscape ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/6df40a30859a7293db9a76fc4fff8cec</t>
         </is>
       </c>
@@ -636,6 +647,11 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>TIDE marsh grass shoot mass (biomass proxy): mean shoot mass per species summed across species per transect; species, creek and branch codes were trimmed of stray whitespace. Reference creeks are West and Nelson; Sweeney (2004-2012) and Clubhead (2005, 2009-2019) were treated as nutrient-enriched only in the years they were fertilized, and other creek-years were dropped.</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
           <t>Deegan, L., Warren, S. &amp; Mozdzer, T. (2022). Data from: “Marsh plant species shoot height, weight and diameters for Rowley River tidal creeks associated with long term fertilization experiments, Rowley and Ipswich, MA. ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/226fb7db2c7b9f8119e40c937b1a19a0</t>
         </is>
       </c>
@@ -699,6 +715,11 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
+          <t>Long-term kelp-removal experiment; annual and continual removal vs. control transects. The missing-value code -99999 was set to missing. Response = summed dry biomass of understory algae and invertebrates (mobile fish and the removed giant kelp excluded). January 2008 surveys, which preceded the first removal, were excluded. Treatments were compared with the control transect at the same reef.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>Reed, D. C. &amp; Miller, R. J. (2024). Data from: “SBC LTER: Reef: Long-term experiment: biomass of kelp forest species, ongoing since 2008 ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/4c63cd36279b7e8448d09651a51ed8a6</t>
         </is>
       </c>
@@ -762,6 +783,11 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
+          <t>Upper Phillips Creek inundation and wrack experiment: wrack was laid over half of each of nine plots in April 1994. The wrack half (transect W) was compared with the no-wrack half (V) of the same plots, 1994-1998; response = live aboveground biomass (species summed per 0.0625 m2 quadrat, x16 to g m-2, quadrats averaged per plot). The package does not identify which plots were flooded, so the inundation treatment was not analyzed.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
           <t>Christian, R. (2019). Data from: “End of Year Biomass for the 1st UPC Inundation Experiment in Upper Phillips Creek marsh 1999-2014 ver 24.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/3854929ce06dc8c667eff9615adb730f</t>
         </is>
       </c>
@@ -825,6 +851,11 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>Tree remeasurement table (TV010 entity 2). Watersheds WS06 (clearcut) and WS07 (shelterwood) vs. control WS08; all live stems (status 1-3) with a measured DBH; mean DBH per plot and census. The control was censused one year after the treatments (2003/2009/2015 vs. 2002/2008/2014); control census years were aligned to the treatment census periods.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
           <t>Franklin, J. F., Bell, D. M., Remillard, S. M., Pabst, R. J., Bluhm, A. &amp; Powers, M. (2025). Data from: “Long-term growth, mortality and regeneration of trees in permanent vegetation plots in the Pacific Northwest, 1910 to present ver 28.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/dc4be3db15934e0e5eb4820f56e5d569</t>
         </is>
       </c>
@@ -888,6 +919,11 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>MELNHE fall litterfall mass per stand; control vs. N, P, NP and Ca. Fertilization began in spring 2011, so 2009-2010 (pre-treatment) were excluded. Treatments were compared with the control plot of the same stand.</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>Yanai, R. D., Fisk, M. C., Vadeboncoeur, M. A., Zukswert, J. M., Mann, T., Young, A., Walsh, G., Morley, M. &amp; See, C. R. (2024). Data from: “Multiple Element Limitation in Northern Hardwood Ecosystems (MELNHE): Litterfall mass 2009-2022 ver 1.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/e2d437bddf1166a733b0df09c87f89f1</t>
         </is>
       </c>
@@ -951,6 +987,11 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
+          <t>Prospect Hill soil respiration (hf005-05). The heated treatment was compared with the disturbance control (cables installed but not heated), which spans the full record; the undisturbed control (1991-2002) was not used. The two June 1991 dates preceding the start of heating were excluded; fluxes were averaged per plot and year.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
           <t>Frey, S. &amp; Melillo, J. (2024). Data from: “Prospect Hill Soil Warming Experiment at Harvard Forest since 1991 ver 37.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/abf59a218a5868baf5b2c073a7dd1d7f</t>
         </is>
       </c>
@@ -1014,6 +1055,11 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
+          <t>Canopy Trimming Experiment soil CO2 flux; block x plot treatment map from the package metadata. The canopy was trimmed between October 2004 and April 2005, so 2003-2004 and the 2005 dates preceding each block's trimming were excluded; chambers were averaged per plot and date.</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>Silver, W. (2023). Data from: “Canopy Trimming Experiment (CTE) trace gases ver 678951.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/97823bf81da5abf22f8f9d8f3778fc58</t>
         </is>
       </c>
@@ -1077,6 +1123,11 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
+          <t>Cascade whole-lake N + P additions: Peter Lake (2013-2015, 2019) and Tuesday Lake (2013-2015) vs. the unmanipulated reference, Paul Lake, in the same years; response = mean manual chlorophyll (carbon proxy) over the sampling season. Lake-years without additions were not paired.</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
           <t>Buelo, C. D., Pace, M. L., Carpenter, S. R., Stanley, E. H., Ortiz, D. A. &amp; Ha, D. T. (2022). Data from: “Cascade Project at North Temperate Lakes LTER – Daily Bloom Data for Whole Lake Experiments 2011 - 2019 ver 2.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5a9862187368b616bed8e20381343717</t>
         </is>
       </c>
@@ -1140,6 +1191,11 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
+          <t>BioCON aboveground biomass, August (peak) harvest only (a June harvest exists only for 1998-2011). The missing-value code 9999 was set to missing; litter and bare-ground records were excluded; plot totals were averaged per ring x treatment. BioCON contains nested designs on different plot sets (main CO2 x N experiment, 4-species 'S' plots, water manipulation from 2007, water x warming from 2012 in the 9-species plots); each treatment was compared with the ambient control of its own design, and those ambient controls were not counted as treatments. Four plots that lost one factor label from 2013 were restored (2) or dropped (2).</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
           <t>Reich, P. (2024). Data from: “Plant aboveground biomass data: BioCON : Biodiversity, Elevated CO2, and N Enrichment ver 13.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/c153c4eb2414bb1ec2ab8b07adc17ef2</t>
         </is>
       </c>
@@ -1203,6 +1259,11 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
+          <t>Compiled herbaceous-biomass table (crop, weeds and cover crops) for the annual cropping systems T1, T2, T3 and T21, with T4 (biologically based, no chemical inputs) as the reference; whole-plant (WHOLE) records were used where reported, so that fractions were not double-counted; litter excluded; stations averaged within replicate and campaigns summed within year. The record begins in 1993, when all systems began to follow one crop sequence; the perennial alfalfa system (T6) was not analyzed.</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
           <t>Robertson, G. &amp; Snapp, S. (2020). Data from: “Annual Net Primary Production on the Main Cropping System Experiment at the Kellogg Biological Station, Hickory Corners, MI (1990 to 2018) ver 85.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f9b2a038b8a7ad43a252587a84935f30</t>
         </is>
       </c>
@@ -1266,6 +1327,11 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
+          <t>Belowground Plot Experiment (burn x mow x nutrient) vs. the unburned, unmowed, unfertilized plots. Response = herbaceous production per 0.1 m2 quadrat (live grass + forbs + current-year dead, which was sorted separately until 2002; woody stems excluded). Quadrats were averaged per plot and date; the two within-year clips of mowed plots were summed, and the last (peak) clip was used for unmowed plots. Treatments were analyzed only while applied: mowing through 2003 and fertilization through 2016.</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
           <t>Blair, J. &amp; Zeglin, L. (2023). Data from: “PBB01 Belowground Plot Experiment: Aboveground net primary productivity of tallgrass prairie based on accumulated plant biomass ver 15.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/d769700c0e40751bfb8b4fb8c34dabb2</t>
         </is>
       </c>
@@ -1329,6 +1395,11 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
+          <t>N fertilization experiment; biomass summed over species within quadrat, quadrats averaged per plot and season; fertilized vs. control plots.</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
           <t>Baur, L., Collins, S., Muldavin, E., Rudgers, J. A. &amp; Pockman, W. T. (2024). Data from: “Nitrogen Fertilization Experiment (NFert): Seasonal Biomass and Seasonal and Annual NPP Data at the Sevilleta National Wildlife Refuge, New Mexico ver 208431.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/9468c8bcda68c0a05c06499ec51b1d55</t>
         </is>
       </c>
@@ -1394,6 +1465,11 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
+          <t>Late-July (peak-season) harvest of each year; aboveground vascular tissues only ('new above' and 'old above'; mosses and lichens were sorted only from 1989, and belowground tissues and litter are excluded); per-quadrat masses of every harvested quadrat scaled to g m-2 (x25) and averaged per block. The 2015 harvest was recovered from the raw quadrat masses. Greenhouse and shade treatments have only two harvests and were not classified.</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
           <t>Shaver, G. (2017). Data from: “Above ground plant biomass in a mesic acidic tussock tundra experimental site from 1982 to 2015 Arctic LTER, Toolik Lake, Alaska. ver 8.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/c3ef07e6ed81c1fc33e9bc20aff07093</t>
         </is>
       </c>
@@ -1457,6 +1533,11 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
+          <t>Half-hourly growing-season NEE from five period files (2009-2021). The 2012 treatment codes (WW/SW) were recoded to those used in other years (W/S). NEE was summed over the season per plot and averaged across the plots of each fence x treatment. Control = ambient winter and summer (C C).</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
           <t>Rodenhizer, H. G., Mauritz, M., Taylor, M., Ledman, J., Natali, S. &amp; Schuur, E. (2022). Data from: “Eight Mile Lake Research Watershed, Carbon in Permafrost Experimental Heating Research (CiPEHR): Half-hourly growing season, chamber-based, CO2 flux data, 2009-2021 ver 23.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/5ee6a71835606934afda8e3eb9a38763</t>
         </is>
       </c>
@@ -1520,6 +1601,11 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
+          <t>Soil CO2 flux after amendment (POST_CO2); water-only (W) plots are the control and C, N, P, CN and CP the treatments (unamended plots were not used). Block numbers are reused in the two lake basins, so a replicate is a basin x block, and treatments were compared with the control of the same basin.</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
           <t>Virginia, R. &amp; Wall, D. (2016). Data from: “McMurdo Dry Valleys Stoichiometry Experiment - CO2 ver 5.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/f2c3854f11c24c54be3f3828c130746f</t>
         </is>
       </c>
@@ -1583,6 +1669,11 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
+          <t>Snow x N x temperature factorial; only ambient-snow, ambient-temperature plots were retained so that the N contrast has an uncontaminated control. Live biomass only (litter is reported separately from 2007; the 2006 harvest did not separate them, so the record begins in 2007).</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
           <t>Suding, K. N., Smith, J. G. &amp; Ashton, I. W. (2024). Data from: “Increased temperature, N and snowpack experiment for north of saddle, 2006 - ongoing. ver 7.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/caacfd0b6e32b5a72f8fe3904ca897bf</t>
         </is>
       </c>
@@ -1645,6 +1736,11 @@
         </is>
       </c>
       <c r="M21" t="inlineStr">
+        <is>
+          <t>Spring annual-plant biomass per 0.25 m2 quadrat, averaged from sub-plot to plot within site; control plot C1 vs. N, P and N+P. 2018 was excluded because 141 of 144 quadrats contained no annual plants.</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>Grimm, N., Hall, S. J., Kaye, J. &amp; Allen, J. (2024). Data from: “Desert Fertilization Experiment: investigation of Sonoran desert ecosystem response to atmospheric deposition and experimental nutrient addition, ongoing since 2006 ver 17.” Environmental Data Initiative. Available at: https://doi.org/10.6073/pasta/fd7e336a9493e780777d97bb08ff2352</t>
         </is>

</xml_diff>